<commit_message>
Add target list: OT ICS IoT
</commit_message>
<xml_diff>
--- a/data/reports/ot-ics-iot.xlsx
+++ b/data/reports/ot-ics-iot.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W27"/>
+  <dimension ref="A1:W26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -619,27 +619,27 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>OT/ICS Cybersecurity Vendor (Software Platform + Services)</t>
+          <t>Pure-play OT/ICS cybersecurity vendor (software platform + professional services)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Hanover, Maryland, United States</t>
+          <t>Hanover, Maryland, USA</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Industrial control systems (ICS)/OT cybersecurity platform and services for electric, oil &amp; gas, manufacturing, water, chemical, mining, transportation, and government sectors</t>
+          <t>Industrial control systems (ICS) / operational technology (OT) cybersecurity across electric, oil &amp; gas, manufacturing, water, chemical, mining, transportation, building automation, food &amp; beverage, pharmaceutical, and government sectors</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>~600-630 employees</t>
+          <t>~600-630 employees (private estimate)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>~$150M-$208M ARR (est., part of newly combined Accenture/Dragos/runZero/NetRise business)</t>
+          <t>$150M-$200M ARR (estimate; 2024 reported at $154.4M ARR)</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -659,27 +659,27 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Dragos is a pure-play, market-leading OT/ICS cybersecurity company whose entire business is industrial threat detection, asset visibility, and OT incident response/consulting services — an ideal target for an OT security consulting/advisory professional.</t>
+          <t>&lt;cite index="1-1"&gt;Dragos provides cybersecurity platforms for operational technology environments, offering asset visibility and threat detection for critical infrastructure.&lt;/cite&gt; &lt;cite index="1-3"&gt;It also offers a suite of assessments including architecture review, device and application vulnerability assessment, network vulnerability assessment, and penetration testing to evaluate and improve OT cybersecurity defenses.&lt;/cite&gt; In mid-2026 &lt;cite index="4-7"&gt;Dragos got acquired by Accenture&lt;/cite&gt;, materially changing its scale, go-to-market, and consulting integration opportunities for OT security talent.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Major inflection event: &lt;cite index="31-2"&gt;Accenture is expanding its position with the acquisition of a majority stake in Dragos and all of runZero and NetRise to deliver end-to-end operational technology (OT) security for the critical infrastructure and industrial operations underpinning power grids, pipelines, manufacturing, distribution facilities and data centers&lt;/cite&gt;. &lt;cite index="32-3"&gt;The deal values industrial cybersecurity giant Dragos at $3.25 billion, and runZero and NetRise will operate under Dragos&lt;/cite&gt;. &lt;cite index="31-6"&gt;Together, Dragos, runZero and NetRise are estimated to generate approximately $208 million in annual recurring revenue as of June 2026, representing 53% year-over-year growth&lt;/cite&gt;. The deal is expected to close August/September 2026, creating significant integration and scaling activity (and likely new roles) as Dragos becomes the OT security platform arm of Accenture's consulting business.</t>
+          <t>&lt;cite index="6-7"&gt;Accenture announced it would take a majority stake and acquire cybersecurity firms in a $4.18 billion deal, including full ownership of runZero and NetRise and majority ownership of Dragos.&lt;/cite&gt; &lt;cite index="4-22"&gt;Dragos also expanded its collaboration with Microsoft to deliver OT-native cybersecurity at global industrial scale, and appointed a new Chief People Officer to support global growth.&lt;/cite&gt; &lt;cite index="4-37"&gt;Dragos also launched EmberAI, an AI assistant addressing the OT security skills gap.&lt;/cite&gt;</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Given the pending Accenture majority-stake acquisition, position outreach around both Dragos' standalone hiring needs and the emerging Accenture-Dragos combined OT security practice; emphasize consulting/advisory experience bridging OT technology and enterprise-scale delivery, since Accenture brings 'decades of trusted relationships' with critical infrastructure operators that will need advisory talent to scale.</t>
+          <t>Engage via Dragos' remote-first careers portal and LinkedIn; given the Accenture majority-stake acquisition, also monitor Accenture's broader industrial/OT cybersecurity practice for combined-entity roles; attend ICS-focused events (S4, BSides ICS) where Dragos is highly visible.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>VP Industrial/OT Cybersecurity Services; Director of Professional Services; Director OT Security Consulting; VP Customer Success - Industrial; Head of Global Services</t>
+          <t>VP Industrial Cybersecurity Services; Director OT Security Consulting; VP Professional Services (ICS/OT); Director Customer Success - OT; Head of OT Security Practice</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Dragos OT cybersecurity; Dragos professional services; Dragos ICS threat intelligence; Dragos Accenture integration; Dragos industrial cybersecurity consultant</t>
+          <t>Dragos OT cybersecurity; Dragos ICS security consultant; Dragos professional services; Dragos Accenture OT security; Dragos industrial cyber threat intelligence</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Active postings found for roles such as Senior ICS/OT Cyber Threat Intelligence Analyst, Senior Cyber Threat Intelligence Analyst (APAC), Data Engineering Manager, Senior Technical Account Manager (OT cybersecurity advisory), and various sales/GTM roles across regions; company describes itself as remote-first and actively recruiting amid the Accenture deal integration.</t>
+          <t>Active open roles found across Dragos' own careers site and job boards (Built In, ZipRecruiter, Indeed, Wellfound) spanning threat intelligence, sales, customer success, engineering, and professional services; &lt;cite index="29-1"&gt;Dragos careers page references Accenture fueling Dragos to build the most complete xOT cybersecurity platform&lt;/cite&gt; as part of ongoing hiring narrative.</t>
         </is>
       </c>
       <c r="R2" t="n">
@@ -702,7 +702,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>https://newsroom.accenture.com/news/2026/accenture-to-strengthen-critical-infrastructure-defense-with-end-to-end-cybersecurity-platform-in-age-of-ai-driven-cyber-threats-and-geopolitical-risk</t>
+          <t>https://www.dragos.com/careers</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -716,47 +716,47 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GuidePoint Security LLC</t>
+          <t>Honeywell International Inc.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.guidepointsecurity.com</t>
+          <t>https://www.honeywell.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Cybersecurity Consulting / VAR / Managed Security Services Provider</t>
+          <t>Diversified industrial conglomerate with dedicated OT cybersecurity product suite and managed services</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Reston, Virginia, United States (also cited as Herndon, VA in some sources)</t>
+          <t>Charlotte, North Carolina, USA</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Broad enterprise and government cybersecurity consulting/advisory, including a dedicated OT Security Services practice (assessments, program development, managed services) alongside cloud, application, identity, and threat/SOC services</t>
+          <t>Process automation, building automation, and industrial control system (ICS) cybersecurity for manufacturing, energy, and critical infrastructure clients globally</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>~1,000-1,150 employees</t>
+          <t>public-company (see EDGAR); reported ~100,000 employees globally</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>~$195M-$267M (estimate; sources vary)</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>estimate</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
+          <t>public-company (see EDGAR)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>public-company (see EDGAR)</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -766,27 +766,27 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>GuidePoint is a large, well-established cybersecurity advisory/consulting firm (not primarily OT-native) that has built out a specific OT security service line, making it a strong fit for OT security consulting expertise even though its core business spans broader IT cybersecurity. &lt;cite index="19-7"&gt;GuidePoint OT Security Services include assessments, program development and managed services to protect critical infrastructure while ensuring uptime and safety.&lt;/cite&gt;</t>
+          <t>&lt;cite index="12-1"&gt;Honeywell announced the expansion of its Operational Technology (OT) Cybersecurity Suite, delivering advanced, proactive protection for industrial environments facing an accelerating wave of sophisticated cyber threats.&lt;/cite&gt; &lt;cite index="16-3,16-4"&gt;Honeywell helps customers keep their environments and assets secure with comprehensive end-to-end cybersecurity solutions, combining professional services, managed security services and its OT Cybersecurity Platform, the Honeywell Cyber Suite.&lt;/cite&gt; This makes Honeywell a large, stable employer for OT security advisory talent with dedicated business units.</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>&lt;cite index="13-6"&gt;More than 6,000 organizations of all sizes and across every industry, as well as over half of U.S. cabinet-level agencies, rely on GuidePoint to strengthen their defenses and reduce risk.&lt;/cite&gt; The firm continues to expand its technology partnerships (e.g., recent partnerships with Netenrich and Specops Software) and was recognized as a Palo Alto Networks 2025 North America Growth Partner of the Year, indicating continued commercial momentum.</t>
+          <t>&lt;cite index="13-1,13-2"&gt;Honeywell introduced Cyber Governance Risk and Compliance (GRC), automating evidence collection and audit reporting through AI and machine learning, as part of an enhanced portfolio to defend critical infrastructure and streamline security compliance.&lt;/cite&gt; &lt;cite index="13-3,13-4"&gt;The company also expanded its managed OT Security Operations Center (SOC) service, providing 24/7 network and endpoint monitoring through a vendor-agnostic platform designed to improve incident response and minimize asset downtime.&lt;/cite&gt; &lt;cite index="17-10"&gt;Honeywell's 2025 Cyber Threat Report found ransomware attacks targeting industrial operators jumped 46% in Q1 2025&lt;/cite&gt;, reinforcing market demand for its OT security offerings.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Target the OT Security Services practice specifically rather than the broader IT security business; emphasize hands-on ICS/SCADA consulting experience since job postings show GuidePoint explicitly seeking candidates with 3+ years in OT security/industrial control systems for pre-sales and delivery roles.</t>
+          <t>Target Honeywell Process Automation and Honeywell Connected Enterprise (HCE) cybersecurity business units; use the June 2026 OT Cybersecurity Suite expansion as a conversation opener; pursue via Honeywell User Group (HUG) events and industrial cyber conferences.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Director OT Security Services; VP Security Consulting Services; Practice Lead - Operational Technology Security; Senior Director Professional Services; VP Solutions Engineering</t>
+          <t>Director OT Cybersecurity Services; VP Cybersecurity, Honeywell Process Automation; Global Sales Director - Cybersecurity; Director Product/Cyber Security (Chief Product Security Leader); Head of OT Security Operations Center</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>GuidePoint Security OT Security Services; GuidePoint Security ICS SCADA; GuidePoint Security operational technology pre-sales; GuidePoint Security security consulting; GuidePoint Security critical infrastructure</t>
+          <t>Honeywell OT cybersecurity; Honeywell Cyber Insights; Honeywell Process Automation cybersecurity; Honeywell HCE cyber security; Honeywell OT SOC</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -796,7 +796,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Active job postings identified for OT-specific roles including a 'Senior Operational Technology Security Pre-Sales Engineer' (remote, anywhere in the U.S.) requiring 3+ years in OT security/ICS/SCADA/IIoT environments, alongside broader ongoing hiring across security engineering, consulting, and federal roles.</t>
+          <t>&lt;cite index="40-8"&gt;Honeywell is currently hiring for 21 open cybersecurity-related positions in the United States per Glassdoor&lt;/cite&gt;, and &lt;cite index="47-1,47-2"&gt;73 Honeywell Cyber Security jobs are listed on Indeed spanning Cybersecurity Engineer, Senior Systems Administrator, and Cybersecurity Analyst roles&lt;/cite&gt;, plus OT-specific postings (e.g., Senior Cyber Security Specialist for Building Automation OT security in the Netherlands).</t>
         </is>
       </c>
       <c r="R3" t="n">
@@ -809,7 +809,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>https://www.indeed.com/q-%22guidepoint-security%22-jobs.html</t>
+          <t>https://www.honeywell.com/us/en/company/ot-cybersecurity</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -833,32 +833,32 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Risk, Safety &amp; Industrial Cybersecurity Consulting (subsidiary of American Bureau of Shipping)</t>
+          <t>Risk, safety, and reliability consulting firm with a dedicated industrial/OT cybersecurity practice</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Spring, Texas, United States</t>
+          <t>Spring, Texas, USA (Houston area)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Risk and reliability engineering consulting for marine/offshore, oil &amp; gas, chemical, power, and industrial sectors, with a dedicated OT/industrial cybersecurity consulting practice and an Industrial Security Operations Center (ISOC)</t>
+          <t>Marine and offshore, oil/gas/chemical, power, government, and industrial manufacturing OT cybersecurity consulting, implementation, and managed services</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1,000-5,000 employees globally</t>
+          <t>1,000+ professionals (ABS Group specifically); part of ABS with 5,000+ employees globally</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>unknown (private subsidiary; no independently disclosed figures found)</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>unknown</t>
+          <t>Unknown (private subsidiary of ABS; no public figures found)</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>estimate</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -866,34 +866,34 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>ABS Group operates a long-standing industrial risk/safety consulting business with a specific OT cybersecurity offering built on deep engineering and critical-infrastructure domain expertise, making it a strong OT-security-adjacent consulting employer for candidates coming from engineering/safety or hybrid IT-OT backgrounds. &lt;cite index="21-27,21-28,21-29"&gt;With more than 50 years of risk and safety management experience, ABS Consulting offers cybersecurity solutions tailored to your operational risk to help you mitigate attacks in real time and minimize operational disruption and downtime... We apply cutting-edge technology targeted to meet your needs and leverage a state-of-the-art Industrial Security Operations Center (ISOC) that allows us to identify and mitigate attacks in real-time&lt;/cite&gt;.</t>
+          <t>&lt;cite index="20-2,20-3"&gt;ABS Group of Companies, Inc. provides data-driven risk and reliability solutions and technical services that help clients confirm the safety, integrity, quality and efficiency of critical assets and operations, operating with more than 1,000 professionals in over 20 countries serving the marine and offshore, oil, gas and chemical, government and industrial sectors.&lt;/cite&gt; &lt;cite index="19-2,19-14"&gt;Its ABS Consulting arm is a premier provider of cybersecurity consulting, implementation, and risk management services grounded in over 50 years of risk and safety management experience.&lt;/cite&gt;</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>&lt;cite index="23-1,23-7"&gt;Headquartered in Spring, Texas, ABS Group operates with more than 1,000 professionals globally, serving the marine and offshore, oil, gas and chemical, government and industrial sectors&lt;/cite&gt; and was named one of America's Best Consulting Firms by Forbes. Regulatory tailwinds are boosting demand: &lt;cite index="28-4,28-5"&gt;the company released a paper to support vessel and facility owners and operators in meeting compliance with the U.S. Coast Guard's (USCG) Maritime Cyber Rule, outlining practical steps to meet the first cybersecurity training deadline of January 12, 2026&lt;/cite&gt;, plus a new MTSA Cybersecurity Training Series product line.</t>
+          <t>&lt;cite index="24-1,24-2"&gt;ABS Consulting expanded its strategic partnership with Dragos to provide industry-leading OT cybersecurity solutions, services and training to federal and commercial organizations, integrating Dragos' technology with ABS Consulting's OT risk management expertise.&lt;/cite&gt; &lt;cite index="24-7,24-8"&gt;ABS Consulting and Dragos are also working with the U.S. Coast Guard on the Maritime Security Risk Analysis Model (MSRAM), creating a near real-time cyber threat/intel tool to evaluate risk to U.S. ports.&lt;/cite&gt;</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Frame outreach around the Cybersecurity/OT practice within ABS Consulting, referencing the maritime cyber regulatory deadline (USCG Maritime Cyber Rule) and ISOC capability as a hook; the firm's engineering/safety heritage means candidates with a blended OT-engineering-plus-cyber background will resonate strongly.</t>
+          <t>Target ABS Group's Cybersecurity Solutions and Global Government consulting divisions; leverage the maritime/MTSA compliance and critical-infrastructure angle; network via ABS's Risk Matters podcast and maritime cybersecurity events.</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Global Head of Industrial Cybersecurity; Director OT Cybersecurity Consulting; Principal Consultant - OT/ICS Security; VP Cybersecurity Solutions; Practice Director - Industrial Security</t>
+          <t>Global Head of Industrial Cybersecurity; Director, Cybersecurity Product Development; VP Cybersecurity Solutions; Principal Consultant, OT Cybersecurity; Director, Government Cybersecurity Consulting</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>ABS Group industrial cybersecurity; ABS Consulting OT cybersecurity; ABS Group ISOC; ABS Consulting maritime cyber; ABS Group cyber risk management</t>
+          <t>ABS Group cybersecurity; ABS Consulting OT cybersecurity; ABS Group industrial cyber; ABS Group ISOC; ABS Consulting maritime cybersecurity</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -903,11 +903,11 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Direct, current OT cybersecurity opening found: &lt;cite index="62-1,62-3,62-4,62-5"&gt;ABS Group is looking for a Principal Consultant to serve as the on-the-ground OT cybersecurity expert for a major industrial client, operating at the intersection of cybersecurity, control systems engineering, and regulatory compliance, advising on ICS/DCS security controls, asset and vulnerability management programs, and MTSA compliance, with a hybrid schedule in southeast Texas&lt;/cite&gt;. Additional related postings include a Telecommunications Analyst supporting IT/OT dependency mapping for DoD clients.</t>
+          <t>&lt;cite index="57-1,57-3"&gt;ABS Group is currently hiring a Principal Consultant to serve as the on-the-ground OT cybersecurity expert for a major industrial client, operating at the intersection of cybersecurity, control systems engineering, and regulatory compliance.&lt;/cite&gt; &lt;cite index="57-4"&gt;The role involves advising on ICS/DCS security controls, strengthening asset and vulnerability management programs, and supporting MTSA compliance efforts.&lt;/cite&gt;</t>
         </is>
       </c>
       <c r="R4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -916,7 +916,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>https://hbbq.fa.us2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1/requisitions</t>
+          <t>https://www.abs-group.com/Solutions/Cybersecurity/</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -930,37 +930,37 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Mangan Inc. (Mangan Cybersecurity)</t>
+          <t>GuidePoint Security LLC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://manganinc.com/ (cyber practice: https://www.mangancyber.com/)</t>
+          <t>https://www.guidepointsecurity.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Boutique OT/ICS engineering &amp; cybersecurity consultancy</t>
+          <t>Cybersecurity Consulting/VAR/MSSP</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Long Beach, California, USA</t>
+          <t>Reston, Virginia, USA</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas, Refining, Pipeline/Midstream, Chemicals &amp; Petrochemical, Biopharma/Life Sciences, Power Distribution</t>
+          <t>Cross-industry cybersecurity solutions/services firm (application security, cloud, IAM, threat intelligence) with a dedicated Operational Technology (OT) security practice serving industrial and critical infrastructure clients alongside Fortune 500 and federal government customers.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>~300-350 employee-owners (private, employee-owned)</t>
+          <t>1,001-5,000 employees (LinkedIn); ~1,000-1,300 per third-party estimators</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>$50M-$150M (estimate)</t>
+          <t>$190M-$270M (estimate; third-party sources vary: Latka ~$194.5M ARR, RocketReach ~$266.9M)</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -968,9 +968,9 @@
           <t>estimate</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -980,41 +980,41 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Mangan runs a dedicated OT cybersecurity brand (Mangan Cybersecurity) built on 31+ years of controls/systems integration experience combined with cyber expertise. Their offering directly matches OT/ICS advisory work: threat and risk analysis, gap analysis, ISA/IEC 62443 alignment, NIST CSF mapping, and their proprietary ICSSbD® toolkit for industrial control system risk assessment.</t>
+          <t>GuidePoint runs a named OT Practice with dedicated OT security engineers/analysts delivering assessments, architecture, and incident response for industrial clients. Its job posting explicitly states it wants candidates with knowledge of &lt;cite index="8-1,8-2"&gt;an in-depth understanding of securing Operational Technology (OT), with knowledge of OT, ICS, SCADA, IIoT, network architecture, and industrial cybersecurity design required.&lt;/cite&gt; The firm also positions itself broadly as &lt;cite index="7-6,7-7,7-8"&gt;a cybersecurity firm offering consulting, engineering, and managed services... with solutions tailored to various platforms including AWS, Microsoft, Google Cloud, and OT environments.&lt;/cite&gt;</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Mangan formalized a strategic partnership with TXOne Networks in 2023 to expand OT cybersecurity hardware/software/services, becoming a certified TXOne systems integrator, indicating active OT security practice expansion alongside their long-standing controls integration business.</t>
+          <t>GuidePoint has repeatedly been recognized as one of Inc. 5000's fastest-growing private companies and describes itself as continuing to expand; a recent posting notes the firm has &lt;cite index="8-12"&gt;grown to over 1,200 employees, established strategic partnerships with leading security vendors, and serves as a trusted advisor to more than 6,200 customers.&lt;/cite&gt;</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Approach via the Mangan Cybersecurity practice leadership rather than the parent engineering firm; emphasize IEC 62443 / ICSSbD-aligned assessment experience and prior refinery/pipeline/chemical OT security engagements to align with their existing client base (oil &amp; gas, TSA Pipeline Directive compliance, chemical terminals).</t>
+          <t>Target the OT Practice leadership and delivery teams directly; emphasize hands-on ICS/SCADA assessment, architecture, and incident-response experience. Use warm intros via GuidePoint's channel partners (e.g., Dragos, Claroty, Xage) mentioned in job postings, and attend GPSEC (GuidePoint's own cybersecurity conference series) for networking.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Chief Technology Officer; Director OT Cybersecurity; VP Industrial Cybersecurity; Practice Lead Cybersecurity Services; Director Controls &amp; Automation</t>
+          <t>Director OT Practice; VP Security Solutions; Director Cybersecurity Advisory; Practice Lead Industrial/OT Security; Senior Manager OT Security Services</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Mangan Cybersecurity; Mangan Inc OT Cybersecurity; ICSSbD Mangan; Mangan Inc controls engineer cybersecurity; Mangan TXOne partnership</t>
+          <t>GuidePoint Security OT Practice; GuidePoint OT Security Engineer; GuidePoint Operational Technology; GuidePoint ICS SCADA; GuidePoint Security Advisory</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Mangan's careers page and LinkedIn/Indeed listings show ongoing recruitment for engineering/controls roles, but no OT-cybersecurity-specific job posting was confirmed as currently open at the time of research; general hiring activity appears active but modest (single-digit open roles reported on job boards).</t>
+          <t>Active/recent postings found for OT-specific roles including 'Operational Technology Security Analyst,' 'Senior Security Engineer, Operational Technology,' and 'Senior Operational Technology Incident Response Engineer' (remote, US), plus a 'Director of Cybersecurity Advisory' role.</t>
         </is>
       </c>
       <c r="R5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>https://www.mangancyber.com/</t>
+          <t>https://www.guidepointsecurity.com/careers/</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -1037,47 +1037,47 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CBIZ Pivot Point Security</t>
+          <t>1898 &amp; Co. (a Burns &amp; McDonnell company)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.pivotpointsecurity.com/</t>
+          <t>https://1898andco.burnsmcd.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>IT/information security compliance consultancy (part of large public professional services firm)</t>
+          <t>Engineering/Consulting firm with dedicated Industrial Cybersecurity practice</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Hamilton/Trenton, New Jersey, USA</t>
+          <t>Kansas City, Missouri, USA</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Cross-industry information security &amp; compliance: technology, healthcare, finance, government, energy, legal (ISO 27001, SOC 2, CMMC, vCISO)</t>
+          <t>Critical infrastructure consulting (energy, utilities, oil &amp; gas, water) with a premier OT/ICS/SCADA cybersecurity consulting practice plus Managed Security Services (MSS) and a dedicated SOC in Houston.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>~30 employees at acquisition (2023); now integrated into CBIZ Technology, LLC (larger parent headcount)</t>
+          <t>Part of Burns &amp; McDonnell, which has 13,500+ employees firm-wide (100% employee-owned); 1898 &amp; Co. itself is a smaller consultancy unit (LinkedIn ~15,600 followers)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Parent is public (CBIZ, NYSE: CBZ) - unit-level revenue not separately disclosed</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>public-company (see EDGAR)</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
+          <t>null - private, employee-owned parent; no standalone financials disclosed</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
@@ -1087,41 +1087,41 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>CBIZ acquired information security consulting firm Pivot Point Security in 2023 to build out cyber/compliance advisory capability. Pivot Point's core services are ISO 27001, SOC audits, penetration testing, vulnerability assessments, vCISO, and CMMC preparation — strong general cybersecurity consulting fit, but public evidence of dedicated OT/ICS-specific practice work is limited; their published focus areas (Kubernetes, DevSecOps, GDPR/CPRA, CMMC) are predominantly IT/compliance rather than industrial/OT.</t>
+          <t>1898 &amp; Co. explicitly operates a &lt;cite index="15-1,15-10"&gt;premier OT/ICS/SCADA cybersecurity consulting practice whose mission is to serve humanity by improving the safety, security, and reliability of the world's critical infrastructure&lt;/cite&gt;, and is &lt;cite index="17-14"&gt;one of the first firms to apply their operational technology (OT) and industrial control systems (ICS) cybersecurity specialization into managed security services.&lt;/cite&gt; It maintains formal technology partnerships for OT security including Claroty, Forescout, and Industrial Defender, and is &lt;cite index="13-14,13-15"&gt;one of a select few private companies partnered to implement Idaho National Labs' (INL) market-leading Consequence-Driven, Cyber-Informed Engineering (CCE) methodology.&lt;/cite&gt;</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>As per a notification letter dated May 12, 2025, the CBIZ Risk &amp; Advisory Services cybersecurity practice (which includes Pivot Point) is being merged with Marcum Technology LLC and rebranded as CBIZ Technology, LLC, effective June 1, 2025 — signaling active consolidation/scaling of CBIZ's broader cybersecurity practice following its 2023 acquisitions.</t>
+          <t>The firm launched a new Managed Threat Protection &amp; Response service built on Dragos, Claroty, and Armis platforms with active response via CrowdStrike, and built a dedicated 24/7 SOC in Houston that started with &lt;cite index="14-19,14-20"&gt;an initial complement of over 60 professionals, choosing Houston because it is central to much of the critical infrastructure, and because the talent pool is large.&lt;/cite&gt; It also recently opened a Cybersecurity Forum and Advanced Threat Protection Center, and continues publishing OT-security thought leadership (e.g., articles from its director of critical infrastructure security consulting).</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Given the 2025 merger into CBIZ Technology, LLC, target the newly combined practice rather than the legacy Pivot Point brand alone; position any pitch around expanding CBIZ Technology's service line into OT/ICS security, an area where the current practice appears to have a gap versus its strong IT/compliance offering.</t>
+          <t>Approach via the Security &amp; Risk Consulting / Managed Security Services leadership team; leverage Burns &amp; McDonnell's employee-ownership culture and long tenure in critical infrastructure engineering as a talking point. Attend or reference 1898 &amp; Co.'s own Cybersecurity Forum / Advanced Threat Protection Center events and OT Cybersecurity Coalition membership for warm networking.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Managing Director Cybersecurity; VP Risk Advisory Services; Practice Leader CBIZ Technology; Director Compliance &amp; Security Consulting</t>
+          <t>Director Industrial Cybersecurity; Director Cybersecurity &amp; Risk Consulting; VP/GM Security Consulting; Director Managed Security Services; Director Advanced Threat Protection Center</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>CBIZ Pivot Point Security; CBIZ Technology cybersecurity; Pivot Point Security ISO 27001; CBIZ Risk Advisory Services cyber; CBIZ CMMC vCISO</t>
+          <t>1898 &amp; Co. OT cybersecurity; 1898 &amp; Co. Industrial Cybersecurity Analyst; Burns &amp; McDonnell ICS security; 1898 &amp; Co. Managed Security Services; 1898 &amp; Co. Security &amp; Risk Consulting</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>No specific current job postings for OT/ICS roles were found; general cybersecurity consulting hiring at CBIZ Technology could not be confirmed as active or inactive from available search results.</t>
+          <t>Job posting found for 'Industrial Cybersecurity Analyst - 1898 &amp; Co. (Washington DC)' supporting IT/ICS security projects (penetration testing, vulnerability assessments, secure system design) using NIST CSF/RMF frameworks; posting noted as remaining open on an ongoing basis until filled.</t>
         </is>
       </c>
       <c r="R6" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1130,7 +1130,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>https://www.pivotpointsecurity.com/company/contact/</t>
+          <t>https://1898andco.burnsmcd.com/what-we-do/industrial-cybersecurity</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1144,42 +1144,42 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1898 &amp; Co. (Burns &amp; McDonnell)</t>
+          <t>Verve Industrial Protection (a Rockwell Automation Company)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://1898andco.burnsmcd.com/</t>
+          <t>https://verveindustrial.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Large engineering-firm-affiliated business/technology/OT security consultancy</t>
+          <t>OT/ICS cybersecurity software &amp; professional services (now integrated product line within a public industrial automation company)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Kansas City, Missouri, USA</t>
+          <t>Originally Paducah, Kentucky, USA (founded as Rkneal Engineering, 1994); now operates as part of Rockwell Automation, headquartered in Milwaukee, Wisconsin</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Critical infrastructure: electric &amp; water utilities, oil &amp; gas refineries/pipelines, transportation, manufacturing — IT/OT convergence, industrial cybersecurity, managed security services</t>
+          <t>OT/ICS endpoint management, asset inventory, vulnerability and patch management for industrial control systems across manufacturing, energy, oil &amp; gas, and utilities; now rebranded under Rockwell's SecureOT suite.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Parent Burns &amp; McDonnell: 13,500+ employee-owners (private, ESOP)</t>
+          <t>Parent company Rockwell Automation employs approximately 29,000 globally; Verve itself was a smaller specialist firm pre-acquisition (headcount not disclosed post-integration)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Parent Burns &amp; McDonnell: est. $7B-$8.9B annual revenue (private, ESOP-owned, no SEC filings)</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>estimate</t>
+          <t>null - Verve's standalone financials not disclosed; parent Rockwell Automation is a publicly traded company (NYSE: ROK) with SEC filings</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>public-company (see EDGAR)</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -1194,41 +1194,41 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>1898 &amp; Co. is explicitly described as a global business, technology and security consultancy serving critical infrastructure industries, and it is a premier OT/ICS/SCADA cybersecurity consulting practice under Burns &amp; McDonnell, offering network penetration testing, vulnerability assessments, secure system design, and NIST CSF/RMF-aligned cybersecurity programs. Its Managed Threat Protection &amp; Response service is one of the first to apply OT/ICS-specialized threat hunting into managed security services, leveraging Dragos, Claroty, Armis, and CrowdStrike partnerships.</t>
+          <t>Verve was a pure-play OT/ICS cybersecurity firm — &lt;cite index="21-2,21-3"&gt;Verve Industrial Protection has ensured reliable and secure industrial control systems for 25 years, with its principal offering, the Verve Security Center, a unique, vendor-agnostic OT endpoint management platform that provides IT-OT asset inventory, vulnerability management, and the ability to remediate threats and vulnerabilities.&lt;/cite&gt; Rockwell Automation completed its acquisition in November 2023, and &lt;cite index="23-15"&gt;Verve will report into Rockwell's Lifecycle Services operating segment.&lt;/cite&gt; The offering has since been rebranded: &lt;cite index="25-15,25-16"&gt;SecureOT™ solution suite is Rockwell Automation's comprehensive industrial cybersecurity offering, bringing together managed and professional services with our OT-specific risk and vulnerability management platform (formerly known as the Verve Security Center), reflecting evolution as a comprehensive, OT‑first cybersecurity partner.&lt;/cite&gt;</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>1898 &amp; Co. joined the Operational Technology Cybersecurity Coalition in 2024 as part of its initial membership expansion, and launched a new Managed Threat Protection &amp; Response capability in 2023 to extend its existing Managed Security Services — both signal active OT-security practice growth. The firm also hosted a dedicated 2024 Cybersecurity Forum and opened an Advanced Threat Protection Center, reflecting continued investment in OT/IT cyber capability.</t>
+          <t>Rockwell continues investing in the platform post-acquisition, with recent launches of enhanced SecureOT capabilities including &lt;cite index="22-3,22-4"&gt;automated patch management and firmware updates for both Rockwell and third-party devices, and advanced analytics for lifecycle management, vulnerability detection, and risk prioritization&lt;/cite&gt;, plus &lt;cite index="22-4"&gt;tiered, modular security services with 24/7 monitoring through Rockwell's global SOC.&lt;/cite&gt;</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Target the Security &amp; Risk Consulting / Advanced Threat Protection Center leadership within 1898 &amp; Co. directly (distinct from core Burns &amp; McDonnell engineering divisions); leverage the firm's active hiring for OT/ICS/SCADA cybersecurity consulting roles and its critical-infrastructure client base (utilities, oil &amp; gas, water, transportation) as an entry point.</t>
+          <t>Since Verve is now fully integrated into Rockwell Automation, target Rockwell's Lifecycle Services / Industrial Cybersecurity business unit rather than a standalone entity. Leverage Rockwell's large customer base and channel/partner ecosystem (e.g., via RSA Conference presence, ManuSec events) for networking, and highlight OT endpoint/vulnerability management expertise relevant to SecureOT.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>VP/General Manager Security &amp; Risk Consulting; Director Advanced Threat Protection Center; Director Cybersecurity &amp; Risk Consulting; Director Managed Security Services; Managing Director OT/ICS Security</t>
+          <t>Director Industrial Cybersecurity (Rockwell Automation); VP Lifecycle Services - Cybersecurity; Director SecureOT Solutions; Practice Lead OT Endpoint Security; Director Managed OT Security Services</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>1898 &amp; Co cybersecurity; 1898 &amp; Co OT ICS security; Burns McDonnell industrial cybersecurity; 1898 &amp; Co Managed Security Services; 1898 &amp; Co Advanced Threat Protection Center</t>
+          <t>Verve Industrial Rockwell Automation; Rockwell Automation SecureOT; Rockwell Automation OT cybersecurity; Verve Security Center; Rockwell Lifecycle Services cybersecurity</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>An Industrial Cybersecurity Analyst role at 1898 &amp; Co. (Washington, DC) was posted in mid-2025 for the OT/ICS/SCADA-focused Security &amp; Risk Consulting practice, indicating active recruiting for OT cybersecurity consulting positions.</t>
+          <t>No standalone Verve careers page found; hiring for OT cybersecurity roles would now fall under Rockwell Automation's broader careers site (not separately verified in this search).</t>
         </is>
       </c>
       <c r="R7" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1237,7 +1237,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>https://1898andco.burnsmcd.com/what-we-do/industrial-cybersecurity</t>
+          <t>https://www.rockwellautomation.com/en-us/capabilities/industrial-cybersecurity/welcome-to-a-new-era-of-ot-security.html</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1251,42 +1251,38 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Nozomi Networks</t>
+          <t>Booz Allen Hamilton</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.nozominetworks.com</t>
+          <t>https://www.boozallen.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>OT/IoT/CPS Cybersecurity Vendor (Network Detection &amp; Response)</t>
+          <t>Large Government/Commercial Consulting &amp; Systems Integrator</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>San Francisco, CA (R&amp;D also in Mendrisio, Switzerland)</t>
+          <t>McLean, Virginia, USA</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Operational Technology (OT), IoT, and cyber-physical systems security platform for critical infrastructure, energy, manufacturing, mining, transportation, utilities, and building automation.</t>
+          <t>Defense, federal civilian, intelligence community, and commercial critical infrastructure (energy, manufacturing, pharma, ports) OT/ICS cybersecurity consulting</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>201-500 employees (estimate)</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>$100M+ ARR (estimate, private/subsidiary reporting)</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>estimate</t>
+          <t>Large (&gt;20,000 employees, public company - see EDGAR)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>public-company (see EDGAR)</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -1301,27 +1297,27 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>&lt;cite index="3-1,3-14"&gt;Nozomi Networks offers a cybersecurity platform that protects operational technology, Internet of Things, and cyber‑physical systems, providing asset discovery, continuous monitoring, threat detection, and risk management.&lt;/cite&gt; As of January 2026, &lt;cite index="41-1,41-3,41-4"&gt;Mitsubishi Electric Corporation completed its acquisition of the company, marking the start of a new phase of growth for Nozomi Networks while preserving the company's independent operations, vendor-neutral technology roadmap, and established go-to-market partnerships, as a wholly owned subsidiary.&lt;/cite&gt; This is a pure-play OT/ICS security vendor -- an excellent fit for OT cybersecurity advisory expertise, though note it now operates as a subsidiary of a large Japanese industrial conglomerate rather than an independent company.</t>
+          <t>Booz Allen runs a dedicated OT Cybersecurity Lab in Chantilly, VA for testing ICS/OT security capabilities, and offers a named OT security methodology (SAF-ICS, built with Splunk) plus a Cyber-Physical Defense practice covering managed OT/ICS SOC-as-a-Service, anomaly detection, and DoD/critical infrastructure engagements. Case studies include a hydroelectric dam and global manufacturers/pharma clients, and it partners with Dragos and Cisco on xOT platforms and live ICS demonstrations at S4 conferences.</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>&lt;cite index="41-5,41-6"&gt;The company recently surpassed $100M in annual revenue and now serves many of the world's largest enterprises, including 5 of the top 10 oil and gas companies, 7 of the top 10 pharmaceutical manufacturers, and 7 of the top 10 utilities.&lt;/cite&gt; &lt;cite index="50-1"&gt;Nozomi has a high compound annual growth rate (CAGR) of 33% and a strong revenue base with a gross profit margin exceeding 70%.&lt;/cite&gt; &lt;cite index="41-10"&gt;It is also cited as the first privately held OT cybersecurity company to achieve sustained cash flow and break-even performance.&lt;/cite&gt; The Mitsubishi Electric deal, valued near $1 billion, is expected to fuel further R&amp;D and go-to-market investment.</t>
+          <t>Booz Allen was recently recognized by Frost &amp; Sullivan as a market leader in Managed Detection and Response, has multiple 2025-2026 published research pieces (AI-driven OT threats, post-quantum crypto-agility, port cyber sabotage risk), and continues publishing new OT thought leadership and live technical demos (e.g., S4x26 industrial security build-out with Cisco).</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Position as an OT cybersecurity advisory partner given its heavy enterprise/critical-infrastructure customer base; target the go-to-market, MSSP/channel, and post-acquisition integration teams (now backed by Mitsubishi Electric) since new investment and joint AI/OT initiatives are underway. Reference Gartner/Forrester leadership recognition when engaging.</t>
+          <t>Target the Cyber-Physical Defense (CPD) and OT Cybersecurity Lab teams directly; reference the SAF-ICS/Splunk offering and Dragos/Cisco partnerships in outreach; leverage conference presence (S4, industrial cyber events) for warm introductions.</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>VP Global Revenue Operations; VP Industrial Cybersecurity; Director OT/ICS Channel &amp; MSSP Programs; Director Professional Services - OT Security; VP Public Sector / Critical Infrastructure</t>
+          <t>VP Cyber-Physical Defense; Director OT/ICS Cybersecurity; Principal OT Security Consulting; Senior Manager Industrial Control Systems Security; Practice Lead Critical Infrastructure Cybersecurity</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Nozomi Networks OT security; Nozomi Networks Mitsubishi Electric; Nozomi Networks MSSP; Nozomi Networks Vantage IQ; Nozomi Networks professional services</t>
+          <t>Booz Allen OT cybersecurity; Booz Allen ICS/SCADA cyber security engineer; Booz Allen cyber-physical defense; Booz Allen critical infrastructure cyber; Booz Allen SAF-ICS</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1331,11 +1327,11 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>&lt;cite index="6-4"&gt;Nozomi Networks is currently seeking a Vice President, Global Revenue Operations.&lt;/cite&gt; General hiring activity continues post-acquisition as the company scales under Mitsubishi Electric ownership.</t>
+          <t>Multiple active OT/ICS-focused postings found, including "OT Cybersecurity Engineer," "OT/ICS Cybersecurity Analyst," "ICS/OT Cyber Security Engineer," and "OT Cybersecurity Analyst" roles across Alexandria, McLean, and remote/DoD-support locations, several requiring Secret/TS-SCI clearance.</t>
         </is>
       </c>
       <c r="R8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1344,7 +1340,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>https://www.nozominetworks.com/press-release/nozomi-networks-enters-next-phase-of-growth-as-mitsubishi-electric-completes-acquisition</t>
+          <t>https://www.boozallen.com/markets/commercial-solutions/operational-technology-ot-cybersecurity-for-business.html</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1358,42 +1354,38 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Claroty</t>
+          <t>Leidos Holdings, Inc.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://claroty.com</t>
+          <t>https://www.leidos.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Cyber-Physical Systems (CPS) / OT-IoT-IoMT Cybersecurity Vendor</t>
+          <t>Large Government/Commercial Systems Integrator &amp; Technology Products</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Reston, Virginia, USA</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Cyber-physical systems protection across industrial (OT), healthcare (IoMT), and enterprise (IoT/Extended IoT) environments, including energy, water, manufacturing, and healthcare sectors.</t>
+          <t>Defense, intelligence, civil government, energy/utilities, oil &amp; gas, nuclear, and manufacturing OT/ICS cybersecurity</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>500-1,000 employees (estimate)</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>$100M-$500M (estimate)</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>estimate</t>
+          <t>Large (&gt;40,000 employees, public company - see EDGAR)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>public-company (see EDGAR)</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -1408,41 +1400,41 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>&lt;cite index="16-1,16-2"&gt;Claroty is the cyber-physical systems (CPS) protection company, founded in 2015 by Team8, headquartered in New York City with global presence across Europe, Asia-Pacific, and Latin America, empowering organizations to secure cyber-physical systems across industrial (OT), healthcare (IoMT), and enterprise (IoT) environments.&lt;/cite&gt; &lt;cite index="16-5"&gt;The company now serves 24 of the Fortune 100 and has been named a Leader in the inaugural Gartner Magic Quadrant for CPS Protection Platforms.&lt;/cite&gt; This is one of the most recognized pure-play OT/CPS security vendors globally, making it a top-tier target for OT cybersecurity advisory expertise.</t>
+          <t>Leidos has a long-standing dedicated Industrial Control Systems practice and owns the Industrial Defender Automation Systems Manager (ASM) product line for ICS asset/configuration/compliance management (NERC CIP, NEI 08-09, NIST SP 800-82). Its Process Control Security Services team includes GICSP-certified engineers with combined decades of OT-only experience across oil &amp; gas, utilities, shipping, nuclear, and manufacturing, and the company operates dedicated ICS R&amp;D/testing labs for power distribution and industrial controller hardware.</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>&lt;cite index="18-2,18-3,18-4"&gt;Claroty announced it has raised $150 million in a Series F funding round led by Golub Growth, an affiliate of Golub Capital, intended to accelerate Claroty's global expansion as it continues to build a comprehensive cybersecurity platform for cyber-physical systems (CPS) and critical infrastructure.&lt;/cite&gt; &lt;cite index="18-6"&gt;Claroty added 24 Fortune 500 customers and recently launched what it described as a first-of-its-kind AI-based catalog for classifying physical assets.&lt;/cite&gt; &lt;cite index="18-6"&gt;The company could be ready for an IPO as early as next year, although that will depend heavily on market conditions.&lt;/cite&gt;</t>
+          <t>Leidos published a 2025 feature on ramping up cyber-physical protection of critical infrastructure, describing AI-powered tools to speed detection of advanced persistent threats on critical infrastructure networks and continued investment in ICS R&amp;D labs.</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Engage via the field/solutions engineering and OT security consulting arms, especially around the Series F growth push into new verticals (healthcare IoMT, federal/public sector). Reference recent Gartner Magic Quadrant Leader status and the CRO change (new Chief Revenue Officer hire) as a conversation starter about expanding advisory/solutions capacity.</t>
+          <t>Approach through the Leidos Cybersecurity / Process Control Security and Industrial Defender product teams; reference NERC CIP/NIST 800-82 compliance expertise and the company's ICS R&amp;D labs; target both the commercial critical-infrastructure business unit and defense-sector cyber-physical teams.</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Chief Revenue Officer; VP OT/ICS Solutions Engineering; Director Professional Services - CPS Protection; VP Federal/Public Sector; Director Threat Research (Team82)</t>
+          <t>Director Industrial Control Systems Security; VP Critical Infrastructure Cybersecurity; Senior Solutions Architect OT/ICS; Practice Lead Process Control Security; Director Cyber-Physical Systems</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Claroty OT security solutions engineer; Claroty xDome; Claroty Team82; Claroty CPS protection; Claroty Series F</t>
+          <t>Leidos ICS cybersecurity; Leidos Industrial Defender; Leidos OT security engineer; Leidos process control security; Leidos critical infrastructure cyber</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Multiple active postings for OT Security Solutions Engineer roles (e.g., Midwest, West regions) found on Claroty's careers site and NightDragon job board; &lt;cite index="53-1,53-2"&gt;LinkedIn currently lists roughly 141 Claroty jobs in the United States.&lt;/cite&gt;</t>
+          <t>No specific current OT/ICS job postings were confirmed in this search snapshot beyond general Leidos cybersecurity capability pages; a dedicated careers-page search for live ICS/OT requisitions is recommended.</t>
         </is>
       </c>
       <c r="R9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1451,7 +1443,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>https://claroty.com/careers</t>
+          <t>https://cyber.leidos.com/solutions/industrial-control-systems</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1465,7 +1457,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Optiv Inc.</t>
+          <t>Optiv Security, Inc.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1475,27 +1467,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Cybersecurity Consulting, Advisory, and Managed Security Services (MSSP)</t>
+          <t>Cybersecurity Solutions Integrator / Advisory &amp; Managed Services</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Denver, CO</t>
+          <t>Denver, Colorado, USA</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>End-to-end cybersecurity strategy, managed security services, incident response, risk &amp; compliance, and security technology integration across virtually every major industry, including critical infrastructure/OT clients.</t>
+          <t>Cross-industry cybersecurity advisory/integration with a dedicated Operational Technology (OT) and IoT security practice serving manufacturing, energy, utilities, and other critical infrastructure clients</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2,000-7,000+ employees (estimate; varies significantly by data source)</t>
+          <t>Mid-large, roughly 1,000-5,000 employees (estimate; sources vary from ~1,600 to ~2,400+)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>$500M-$1B+ (estimate; private company, figures vary widely across data providers)</t>
+          <t>$500M-$1.5B (estimate; third-party estimates vary widely and are not SEC-verified since Optiv is privately held)</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1515,27 +1507,27 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>&lt;cite index="24-6,24-7"&gt;Optiv is the cyber advisory and solutions leader, delivering strategic and technical expertise to nearly 6,000 companies across every major industry, partnering with organizations to advise, deploy and operate cybersecurity programs from strategy and managed security services to risk, integration and technology solutions.&lt;/cite&gt; As one of the largest independent cybersecurity consulting/advisory firms in North America, Optiv is a strong target for OT cybersecurity advisory talent, though OT/ICS is one practice area within a much broader IT-security consulting portfolio rather than its sole focus.</t>
+          <t>Optiv operates a named OT/IoT security practice offering advisory, deployment, and managed services (including an OT Security Operations Center/Advanced Fusion Center) specifically for SCADA, PLC, and ICS environments, led by a dedicated Practice Director for OT/IoT. The practice was formally launched/expanded with a full suite of OT security services and has been featured in Gartner's Market Guide for Operational Technology Security.</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Optiv previously filed for an IPO (S-1, 2016) but withdrew the registration in 2018 and remains privately held (previously backed by private equity including KKR and Blackstone per historical reporting). &lt;cite index="35-2,35-9"&gt;As of mid-2026, Optiv is actively hiring for around 29 open positions in the United States according to Glassdoor.&lt;/cite&gt; The company continues to run its annual 'OptivCon' industry event and produce cyber-risk thought leadership content, signaling ongoing market engagement.</t>
+          <t>Optiv publicly launched its full suite of OT security advisory, deployment, and management services and continues to market OT/IoT-specific advisory and managed SOC offerings; Optiv states its advisors deliver expertise to nearly 6,000 client companies, reflecting a broad and growing consulting client base.</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Target Optiv's advisory/consulting practice leads and industrial/critical-infrastructure vertical teams; given its broad generalist cyber consulting client base, position OT expertise as a differentiator to help Optiv expand its OT/ICS advisory offering. Look for practice-level or 'Principal Advisor' roles focused on industrial clients.</t>
+          <t>Engage the OT/IoT practice directly (referencing the OT Security Operations Center / Advanced Fusion Center offering); target Optiv's infrastructure &amp; cloud security business unit leadership; leverage Optiv's stated OT advisor tenure (nearly 130 combined years of on-the-ground ICS experience) as a hook for peer-to-peer networking.</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>VP Industrial/OT Cybersecurity Practice; Principal Advisor - Critical Infrastructure; Director OT/ICS Security Consulting; VP Advisory Services; Practice Director - Risk &amp; Compliance</t>
+          <t>Practice Director OT/IoT Security; VP Infrastructure &amp; Cloud Security; Principal Cybersecurity Advisor - OT/ICS; Director Product Security - ICS/IoT; Senior Manager OT Security Services</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Optiv OT security consulting; Optiv critical infrastructure advisory; Optiv Principal Cybersecurity Advisor; Optiv managed security services; Optiv ICS SCADA</t>
+          <t>Optiv OT security; Optiv ICS/IoT practice; Optiv operational technology advisor; Optiv OT SOC; Optiv critical infrastructure cybersecurity</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1545,11 +1537,11 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>&lt;cite index="35-2"&gt;Optiv is currently hiring for 29 open positions in the United States per Glassdoor&lt;/cite&gt;; &lt;cite index="34-1"&gt;Indeed lists 23 Optiv Cyber Security jobs available&lt;/cite&gt;, spanning advisory, engineering, and sales roles, though no OT-specific listings were confirmed at time of research.</t>
+          <t>Active listings found for various cybersecurity advisor/consultant roles (e.g., Principal Cybersecurity Advisor, Senior Cybersecurity Advisor - Security Operations, Senior Consultant - Cybersecurity) though no OT-specific requisition was directly confirmed in this snapshot; general cybersecurity consulting hiring activity is ongoing.</t>
         </is>
       </c>
       <c r="R10" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -1558,7 +1550,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>https://www.optiv.com/company/careers</t>
+          <t>https://www.optiv.com/services/infrastructure/operational-technology</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1572,7 +1564,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ampyx Cyber</t>
+          <t>Ampyx Cyber (formerly Ampere Industrial Security)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1582,27 +1574,27 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>OT/ICS Cybersecurity Consulting Firm (Pure-Play)</t>
+          <t>Boutique OT/ICS cybersecurity consulting firm</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Portland, Oregon, USA (also Tallinn, Estonia office; registered entities in US and Germany)</t>
+          <t>Portland, Oregon, USA (also operates in Tallinn, Estonia and Germany)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Critical infrastructure asset owners — power/electric utilities, water, gas, transportation; deep NERC CIP, NIS2, CER, and Cyber Resilience Act (CRA) regulatory focus</t>
+          <t>Critical infrastructure (electric utilities, water, gas, transportation) — NERC CIP, NIS2, CRA regulatory compliance</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Small (estimate, ~20-75 employees)</t>
+          <t>Small (estimate, likely &lt;50 people; largely 1099/remote consultant model)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>$5M-$25M (estimate)</t>
+          <t>&lt;$10M-$25M (estimate)</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1622,27 +1614,27 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Ampyx Cyber (formerly Ampere Industrial Security) is a services-only firm exclusively focused on ICS/OT security and regulatory compliance. Its own materials state it is &lt;cite index="3-1,3-2"&gt;a specialized, services-only international consulting firm operating across North America and Europe, focused exclusively on the security of Industrial Control Systems (ICS) and Operational Technology (OT)&lt;/cite&gt;, with offerings including &lt;cite index="3-11,3-12,3-13,3-14,3-15"&gt;regulatory compliance &amp; strategy in NERC CIP, NIS2, CER, and CRA frameworks, gap audits, vulnerability assessments, M&amp;A diligence, OT Zero Trust implementation, network segmentation, hardening, supply chain security, and specialized IT/OT training&lt;/cite&gt;. This is one of the most pure-play OT security consultancies on the target list.</t>
+          <t>Ampyx Cyber is a specialized, services-only consulting firm exclusively focused on ICS/OT security and regulatory compliance for critical infrastructure asset owners. Its core team includes former utility staff, standards drafters, and federal auditors — a strong match for an OT cybersecurity advisory professional.</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>The firm recently rebranded and expanded internationally: &lt;cite index="8-9,8-10"&gt;'As we transition to Ampyx Cyber, we're not only redefining our brand but also expanding our global footprint,' with new offices in Portland and Tallinn signaling growing international reach&lt;/cite&gt;. It also &lt;cite index="3-7"&gt;appointed a new Chief Revenue Officer, Andrew Luccitti, to push growth and innovation in industrial cybersecurity&lt;/cite&gt;, and is actively publishing threat commentary (e.g., on Volt Typhoon) signaling market visibility efforts.</t>
+          <t>The company rebranded from Ampere Industrial Security to Ampyx Cyber and has been actively expanding its international footprint, including opening a new office in Tallinn, Estonia, alongside its Portland base, and recently appointed a new Chief Revenue Officer to drive growth.</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Approach via the engagement/business development team listed on the site; highlight NERC CIP/utility sector experience and hands-on OT pentesting delivery skills; reference the firm's stated hiring philosophy valuing deep industry/regulatory expertise over corporate hierarchy.</t>
+          <t>Approach as a niche, high-trust boutique consultancy; emphasize deep OT/ICS/NERC CIP domain expertise and independence from vendor influence (technology-agnostic positioning) in outreach. Reference specific service lines (RAPID OT assessments, NERC CIP compliance, supply chain security) to show fit.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Chief Revenue Officer; VP Industrial Cybersecurity Consulting; Director OT/ICS Security Practice; Practice Lead NERC CIP Compliance</t>
+          <t>Chief Revenue Officer; VP Consulting Services; Director OT/ICS Security Practice; Practice Lead Industrial Cybersecurity</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Ampyx Cyber; Ampere Industrial Security; OT ICS security consultant NERC CIP; industrial cybersecurity Portland Oregon</t>
+          <t>Ampyx Cyber; Ampere Industrial Security; OT/ICS consulting Portland; NERC CIP consultant; industrial cybersecurity consulting firm</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1652,11 +1644,11 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>No explicit current job postings were found in search results; however the company messaging emphasizes recruiting 'a different kind of expert' and recent growth/CRO hire suggests possible expansion hiring.</t>
+          <t>The firm maintains a 'Current Openings' page inviting resumes on a rolling basis for a remote, 1099 contractor consulting model rather than posting specific formal job requisitions, so it's unclear if there are active open roles at any given time.</t>
         </is>
       </c>
       <c r="R11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
@@ -1679,37 +1671,37 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AcuTech Group, Inc. (AcuTech Consulting Group)</t>
+          <t>UTSI International Corporation</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://acutech-consulting.com</t>
+          <t>https://utsi.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Process Safety, Security &amp; Emergency Management Consulting Firm (with OT/ICS Cybersecurity Practice)</t>
+          <t>OT/ICS systems integration, engineering, and cybersecurity consulting firm</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Virginia, USA (also offices in India, Asia-Pacific, Europe, and the Middle East)</t>
+          <t>Houston, Texas, USA (corporate office also listed in Friendswood, TX)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Chemical, petrochemical, oil &amp; gas, refining, pharmaceutical, LNG, hydrogen, and anhydrous ammonia industries — core focus is process safety/PSM with a dedicated Functional Safety &amp; ICS Cybersecurity Services group</t>
+          <t>Oil &amp; gas pipelines, SCADA/ICS engineering, energy and critical infrastructure OT cybersecurity</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Mid-size (estimate, ~100-300 employees globally)</t>
+          <t>Small (estimate; third-party sources vary from ~16 to ~50 employees)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>$20M-$75M (estimate)</t>
+          <t>$1M-$25M (estimate; third-party estimates vary widely)</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1717,53 +1709,53 @@
           <t>estimate</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Medium-High</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>AcuTech is &lt;cite index="11-2,11-3"&gt;a global leader providing best-in-class consulting, training, and software solutions to manage process risk, operating since 1994&lt;/cite&gt;, and explicitly lists &lt;cite index="13-2"&gt;Cybersecurity for Industrial Control Systems as one of its priority service areas&lt;/cite&gt; alongside process safety and functional safety. The firm maintains a dedicated &lt;cite index="16-1"&gt;Functional Safety &amp; ICS Cybersecurity Services group&lt;/cite&gt;, and its security service line states &lt;cite index="15-3"&gt;seasoned consultants bring expertise in Operational Technology/Industrial Control Systems (OT/ICS) cybersecurity, with a focus on conducting thorough audits&lt;/cite&gt;. This makes it a strong adjacent-fit target where OT cyber is a growing practice within a larger process-safety brand.</t>
+          <t>UTSI International has focused on SCADA/ICS engineering and OT cybersecurity consulting for the pipeline and critical infrastructure sector for four decades, and has been recognized as a Top OT Cybersecurity Consultant for 2025, making it directly relevant to an OT security consulting career.</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>The company states &lt;cite index="13-1,13-13"&gt;this investment has enabled sustained global growth through targeted expansion of teams and capabilities, and AcuTech plans to expand its global network of consultants&lt;/cite&gt;, and is actively recruiting broadly: &lt;cite index="11-20"&gt;'We are continually searching for individuals to contribute to our core business, expand our presence in growing markets, and augment our service portfolio.'&lt;/cite&gt; It also had a strong presence at the 2026 AIChE/GCPS conference presenting on cybersecurity for industrial control systems alongside process safety topics.</t>
+          <t>UTSI reports consistent double-digit year-over-year growth for three consecutive years, has acquired Pandata Tech to add AI/ML capability, formed an OT Cybersecurity Advisory Board, secured a two-year U.S. Space Force contract, and recently announced a strategic partnership/joint venture with Quantum River.</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Target the Functional Safety &amp; ICS Cybersecurity Services group leadership directly; position candidate as complementary hire to grow the cybersecurity practice beyond its process-safety roots; engage via conference presence (AIChE/GCPS) and LinkedIn.</t>
+          <t>Position as a smaller, growth-stage OT engineering/cyber consultancy with deep pipeline/SCADA legacy; emphasize hands-on ICS/SCADA and NERC CIP/IEC 62443 experience plus familiarity with tools UTSI partners with (Nozomi, Fortinet, ThreatGEN, Frenos, Axio, BlastWave) when reaching out.</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Group Leader Functional Safety &amp; ICS Cybersecurity Services; Director of Security Consulting; VP Process Safety &amp; Security; Principal Consultant OT/ICS Cybersecurity</t>
+          <t>President; VP Operations &amp; Strategy; OT Cybersecurity Lead; Director ICS/SCADA Consulting</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>AcuTech Consulting Group; AcuTech Group Inc; ICS cybersecurity process safety; CFATS security vulnerability assessment consultant</t>
+          <t>UTSI International; UTSI OT cybersecurity; SCADA pipeline cybersecurity consultant; ICS engineering Houston; OT Cybersecurity Advisory Board UTSI</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>Company site actively solicits applicants to expand its service portfolio and growing markets; recent global expansion into India, APAC, Europe, and Middle East offices suggests ongoing headcount growth.</t>
+          <t>No specific current job openings were found on UTSI's own site or major job boards during this search; Indeed reviews reference historically high turnover, but no confirmed active postings were located.</t>
         </is>
       </c>
       <c r="R12" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1772,7 +1764,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>https://acutech-consulting.com/about/</t>
+          <t>https://utsi.com/</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1786,37 +1778,37 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Aerstone</t>
+          <t>Claroty, Inc.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://aerstone.com</t>
+          <t>https://claroty.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Cybersecurity Consulting &amp; Assessment Firm (NSA-Certified Vulnerability Assessor; Federal + Commercial, with OT/Utilities practice)</t>
+          <t>OT/ICS and cyber-physical systems (CPS) cybersecurity product vendor</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Rockville, Maryland / Springfield, Virginia, USA (also Boulder, Colorado)</t>
+          <t>New York, New York, USA (with offices in Israel, Europe, Asia-Pacific, Latin America)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Federal government, military, and intelligence community clients plus commercial sectors (financial services, healthcare, utilities, aerospace, education); dedicated OT/ICS cybersecurity offering for electric, gas, and pipeline utilities</t>
+          <t>Industrial (OT), healthcare (IoMT), and enterprise IoT — the 'Extended Internet of Things (XIoT)' across manufacturing, energy, healthcare, and public sector</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Small (estimate, ~20-50 employees)</t>
+          <t>Mid-size (estimate; third-party sources put headcount roughly in the 250-1,000 range depending on source)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>$5M-$20M (estimate)</t>
+          <t>Estimated in the $150M-$300M+ ARR range per third-party sources (private company; precise SEC-verified figures not applicable as Claroty is not currently public)</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1824,9 +1816,9 @@
           <t>estimate</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
@@ -1836,27 +1828,27 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Aerstone is &lt;cite index="24-4"&gt;an NSA-Certified Vulnerability Assessor (NSA VAS) and Service-Disabled Veteran-Owned Small Business (SDVOSB) that provides subject matter expertise in the field of advanced cybersecurity&lt;/cite&gt;, and has built out a specific OT/ICS practice for utilities: &lt;cite index="21-1,21-2"&gt;Aerstone's OT Cybersecurity Assessments help utilities and critical-infrastructure operators establish a precise baseline of control-system security, backed by a cleared team of subject matter experts in operational technology (OT), industrial control systems (ICS), and energy sector compliance&lt;/cite&gt;. Its offerings explicitly cover &lt;cite index="21-9"&gt;TSA pipeline security directives, DHS/CISA guidance (including VADR), and NERC CIP&lt;/cite&gt;, making it a genuine (if smaller/boutique) OT cybersecurity consulting target.</t>
+          <t>Claroty is a leading dedicated OT/CPS cybersecurity vendor, launched by the Team8 foundry in 2015 and headquartered in New York with a global presence, and has been named a Leader for the second consecutive year in the 2026 Gartner Magic Quadrant for CPS Protection Platforms — making it a top-tier target for OT cybersecurity professionals given its scale and market leadership.</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>The firm is expanding OT-specific service lines (VADR for pipeline operators, OT architecture design, SCADA/ICS penetration testing) and is actively hiring across cybersecurity roles: &lt;cite index="32-17"&gt;Yes, Aerstone has 6 open jobs&lt;/cite&gt;, and its LinkedIn page notes &lt;cite index="31-14,31-15,31-16"&gt;Aerstone is hiring! seeking an experienced cybersecurity tester to join a test team supporting security control-based application, networking, mobile, and cloud-based penetration testing&lt;/cite&gt;.</t>
+          <t>Claroty recently secured $150 million in Series F funding led by Golub Growth, has raised over $700 million in total investment with roughly $300 million in annual recurring revenue over the past three years, and continues to expand its Public Sector practice and partner ecosystem (e.g., AWS Strategic Collaboration Agreement).</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Engage via careers page/Indeed postings and LinkedIn; emphasize NSA VAS credential alignment and TSA/NERC CIP utility compliance experience; position toward growing the newer OT/critical-infrastructure practice specifically.</t>
+          <t>Given its size and Gartner Leader status, target Claroty for roles spanning sales engineering, professional services, public sector, and channel/partnerships; leverage its named research arm (Team82) and platform (xDome, Continuous Threat Detection) in conversations to demonstrate familiarity with their offerings.</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>CTO; Director OT/ICS Security Services; VP Critical Infrastructure Cybersecurity; Practice Lead SCADA/Utilities Security</t>
+          <t>VP Professional Services; Director Industrial/OT Security Practice; VP Public Sector; Regional Sales Director - Industrial Cybersecurity; Director Solutions Engineering</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Aerstone cybersecurity; Quest Consultants LLC Aerstone; NSA certified vulnerability assessor OT; Aerstone utilities cybersecurity</t>
+          <t>Claroty; Claroty industrial cybersecurity; Claroty OT security; Claroty Team82; Claroty xDome; Claroty Public Sector</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1866,11 +1858,11 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>Indeed lists 6 open jobs at Aerstone (Springfield, VA and Washington, DC roles including Senior Cybersecurity Analyst, Penetration Tester, Back-End/Front-End Developer); LinkedIn also shows active hiring posts for penetration testing roles.</t>
+          <t>Claroty's careers page and multiple job boards (LinkedIn, ZipRecruiter, Built In) show active, ongoing hiring across roles including Customer Success Manager, Professional Services Engineer, Technical Account Manager, Public Sector sales, Sales Development Representatives, and FedRAMP Compliance Analyst.</t>
         </is>
       </c>
       <c r="R13" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -1879,7 +1871,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>https://aerstone.com/utilities-cybersecurity/</t>
+          <t>https://claroty.com/careers</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1893,37 +1885,37 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>UTSI International Corporation</t>
+          <t>Nozomi Networks, Inc.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://utsi.com/</t>
+          <t>https://www.nozominetworks.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>OT/ICS Cybersecurity &amp; SCADA Systems Integrator (boutique consultancy)</t>
+          <t>OT/ICS Cybersecurity Vendor</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Houston/Friendswood, TX, USA</t>
+          <t>San Francisco, California, USA</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Oil &amp; gas pipelines, energy, transportation, critical infrastructure SCADA/ICS engineering and OT cybersecurity consulting</t>
+          <t>Operational technology (OT), IoT, and cyber-physical systems (CPS) security platform provider serving critical infrastructure, energy, manufacturing, mining, transportation, building automation, water/wastewater, healthcare and other industrial sectors.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>11-50 (estimate)</t>
+          <t>300-400 employees (est.)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>$5M-$25M (estimate)</t>
+          <t>~$62.5M (2023) → ~$74.7M (2024) → ~$101.7M (2025) net revenue</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1943,41 +1935,41 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>UTSI is a boutique systems integrator with over four decades of pipeline/SCADA engineering roots that has pivoted heavily into OT/ICS cybersecurity consulting. The company positions itself as an OT cybersecurity solution provider offering risk assessments, incident response planning, tabletop exercises, and regulatory compliance services for critical infrastructure operators. It has been recognized as a top OT cybersecurity consultancy and works with Fortune 500 OT asset owners.</t>
+          <t>Nozomi Networks is a pure-play OT/IoT/ICS cybersecurity vendor, widely regarded as a market leader in industrial cybersecurity visibility, threat detection and asset intelligence — a strong culture and product fit for an OT security consultant/advisor.</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>UTSI has been actively expanding partnerships (Nozomi Networks, Fortinet, Schneider Electric, ThreatGEN, Quantum River) and recently announced a strategic partnership and joint venture, plus a two-year U.S. Space Force contract. The company was recognized as 'Top OT Cybersecurity Consultants 2025' by Cyber Security Review Magazine, and has built an internal SCADA R&amp;D lab and AI tooling (DANN2.0) for OT.</t>
+          <t>Nozomi Networks was acquired by Mitsubishi Electric, with the deal fully completed around January 29, 2026, following prior minority investment; Mitsubishi Electric's press materials show net revenue growing from $62.56M (2023) to $101.7M (2025). The company continues to expand its platform (e.g., Vantage, Guardian Air, Arc) and recently launched Guardian and Central Management Console on Google Cloud Marketplace, and formed new alliances (e.g., with the UAE Cybersecurity Council and Open Systems in EMEA).</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Approach as a boutique/growing OT cybersecurity consultancy expanding its advisory bench strength; position around pipeline/energy sector expertise, NERC CIP/IEC 62443 frameworks, and executive/board-level cyber risk communication capabilities given their emphasis on translating technical risk into board presentations.</t>
+          <t>Target via Nozomi's professional services, MSSP partner, and channel teams, since much OT consulting/advisory work flows through their Designated Engineer and Fast Track Services programs and MSSP Elite Program; leverage the recent Mitsubishi Electric acquisition and integration activity as a conversation starter around expanded industrial security service delivery needs.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>President/CEO; VP Operations &amp; Strategy; Director OT Cybersecurity Services; Senior Cybersecurity Consultant OT/IT</t>
+          <t>VP Professional Services; Director OT Security Services; Head of Customer Success - Industrial; VP Channel &amp; Alliances; Director Solutions Engineering</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>UTSI International OT cybersecurity; UTSI International ICS SCADA consultant; UTSI International pipeline cybersecurity; UTSI Houston critical infrastructure</t>
+          <t>Nozomi Networks professional services; Nozomi Networks OT security consultant; Nozomi Networks solutions engineer; Nozomi Networks MSSP; Nozomi Networks Mitsubishi Electric integration</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>No specific current OT cybersecurity job openings were found in search results; general employer review pages (Indeed/Zippia) exist but do not show live cybersecurity-specific postings at research time.</t>
+          <t>Active listings include Account Manager, Sales Engineer, Senior Sales Engineer, Associate Customer Success Manager, and other GTM/technical roles per Built In and ZipRecruiter listings; company career site actively promotes open positions.</t>
         </is>
       </c>
       <c r="R14" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
@@ -1986,7 +1978,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>https://utsi.com/</t>
+          <t>https://www.mitsubishielectric.com/en/pr/2026/pdf/0129.pdf</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -2000,38 +1992,38 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Xage Security</t>
+          <t>IBM Corporation (IBM Consulting)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://xage.com/</t>
+          <t>https://www.ibm.com/services/ot-security</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>OT/IT/Cloud Zero Trust Cybersecurity Vendor</t>
+          <t>Global IT/Professional Services &amp; Consulting (OT Security Practice)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Palo Alto, California, USA</t>
+          <t>Armonk, New York, USA</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Energy, utilities, defense, manufacturing, oil &amp; gas, logistics/supply chain, and critical infrastructure zero-trust access and identity security</t>
+          <t>Enterprise-wide cybersecurity consulting and managed services including a dedicated OT security practice covering assessment, protection, and OT SOC services for industrial, critical-infrastructure and asset-intensive clients across energy, utilities, manufacturing, transport and other regulated sectors.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>~112 employees (estimate, per Tracxn)</t>
+          <t>250,000+ employees (large public multinational)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>estimate</t>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>public-company (see EDGAR)</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -2046,27 +2038,27 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Xage is a leading vendor in zero-trust access control purpose-built for OT, IT, and cloud environments, serving critical infrastructure customers like Kinder Morgan and the U.S. Space Force. It also runs a dedicated Xage Cybersecurity Services practice offering OT risk management and consulting, which directly overlaps with OT security advisory work.</t>
+          <t>IBM Consulting operates a formal OT Security Services line offering assessment, protection, and OT SOC deployment services, with named consulting roles such as "Senior Managing Consultant - OT Cybersecurity" and partnerships with Nozomi, Claroty, ABB, and Palo Alto Networks — making it a direct, high-scale target for an OT cybersecurity advisory professional.</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Xage has raised a total of $80M over 6 rounds, including a Series B round completed in December 2025, and reported 112 employees as of May 2026. Recent momentum includes a partnership with LTIMindtree for zero trust in critical infrastructure, integration with NVIDIA BlueField/DOCA for AI security, a Forescout partnership, and a $1.5M U.S. Navy contract for zero trust initiatives.</t>
+          <t>IBM's OT security page cites that in 2023, 70% of industrial organizations experienced a cyberattack, and highlights IBM's X-Force Threat Intelligence Index and expanding partner ecosystem (Microsoft, Palo Alto Networks, Claroty, Nozomi MSSP Elite Program) as part of its OT security push. IBM Consulting Advantage for Cybersecurity, a new AI-powered unified security platform, was also recently introduced to bring together disparate security technologies including OT.</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Target as a fast-growing zero-trust/OT security vendor actively expanding its services and federal/critical-infrastructure business; emphasize consulting/advisory experience that complements their Xage Services professional services arm and federal government practice.</t>
+          <t>Approach via IBM Consulting's Cybersecurity Services practice leads and regional OT/industrial security practice leaders; reference specific open roles like "Senior Managing Consultant - OT Cybersecurity" and "Cyber Security Consultant - Operational Technology (OT)" as evidence of active practice-building and hiring need for senior OT talent.</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Chief Revenue Officer; VP Federal Sales; SVP Solutions Advisory &amp; Customer Success; Director OT/Industrial Cybersecurity Services</t>
+          <t>Senior Managing Consultant OT Cybersecurity; Global Practice Leader OT/ICS Security; Partner Cybersecurity Services; Director Industrial Security Consulting; OT Security Specialist Lead</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Xage Security OT cybersecurity; Xage Security zero trust critical infrastructure; Xage Security services consultant; Xage Security federal</t>
+          <t>IBM Consulting OT security; IBM X-Force ICS; IBM OT cybersecurity consultant; IBM Consulting Advantage Cybersecurity; IBM industrial control systems security</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -2076,11 +2068,11 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>Multiple job boards show active openings (Indeed lists 7 jobs, ZipRecruiter lists 6, Glassdoor lists 7), including engineering, solutions architect, and go-to-market roles.</t>
+          <t>Multiple current job postings found for OT-specific consulting roles, including 'Senior Managing Consultant - OT Cybersecurity' (KSA/MEA region, requiring 10-12 years OT security leadership experience) and 'Cyber Security Consultant - Operational Technology (OT)' roles in the UK, indicating active practice expansion.</t>
         </is>
       </c>
       <c r="R15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
@@ -2089,7 +2081,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>https://xage.com/</t>
+          <t>https://www.ibm.com/services/ot-security</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2103,42 +2095,42 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Verve Industrial Protection (a Rockwell Automation Company / SecureOT)</t>
+          <t>Forescout Technologies, Inc.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://www.rockwellautomation.com/en-us/capabilities/industrial-cybersecurity/welcome-to-a-new-era-of-ot-security.html</t>
+          <t>https://www.forescout.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>OT Cybersecurity Software &amp; Services (subsidiary of public industrial automation company)</t>
+          <t>OT/IoT/IT Cybersecurity Vendor (Asset Visibility &amp; NAC)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Milwaukee, Wisconsin, USA (Rockwell Automation parent HQ); Verve originally Chicago, IL-based</t>
+          <t>San Jose, California, USA</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Manufacturing, critical infrastructure, and industrial automation OT asset inventory, vulnerability management, and managed cybersecurity services</t>
+          <t>Agentless cybersecurity platform delivering asset visibility, network access control, risk/exposure management, and threat detection/response across IT, IoT, IoMT, and OT device types, serving Fortune 100 enterprises and government agencies.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Public company (see EDGAR) — Rockwell Automation parent employs approximately 29,000 globally</t>
+          <t>~1,000-1,300 employees (est.)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Public company (see EDGAR)</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>public-company (see EDGAR)</t>
+          <t>~$189M-$710M (estimates vary widely across data providers; treat as estimate only)</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>estimate</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -2153,27 +2145,27 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Rockwell Automation acquired Verve Industrial Protection in 2023, and Verve's asset inventory, vulnerability management, and patch/configuration management platform now underpins Rockwell's SecureOT suite. This is a leading, well-resourced OT cybersecurity practice with deep consulting service offerings, backed by a Fortune 500 parent that is the world's largest industrial automation company.</t>
+          <t>Forescout is a well-established cybersecurity vendor whose platform explicitly covers OT/ICS visibility and network segmentation as part of its Enterprise of Things/asset security suite, with dedicated Professional Services Engineer roles that involve OT/ICS deployment consulting — a good fit for an OT cybersecurity advisory candidate.</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>In June 2026, Rockwell Automation launched three enhanced offerings within the SecureOT suite, adding managed services and AI/ML-driven assessment capabilities, and highlighted its IEC 62443-4-1 Maturity Level 4 certification. Rockwell continues to post OT cybersecurity consultant, sales executive, and security architect roles across multiple locations, reflecting continued investment in the practice.</t>
+          <t>Forescout was taken private by Advent International (with Crosspoint Capital Partners as co-investor) in 2020 in a deal valued at $1.9 billion, and remains under private equity ownership as of 2025-2026, pursuing continued acquisitions and expansion into the roughly $25 billion OT security market; the company has also recently made executive changes including a new Chief Revenue Officer and VP of Product Marketing.</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Engage via Rockwell's Lifecycle Services / SecureOT organization; position experience with NIST CSF, IEC 62443, NERC CIP, and MITRE ATT&amp;CK for ICS frameworks, and target the OT cybersecurity consulting/advisory teams that serve Fortune 1000 manufacturing clients.</t>
+          <t>Target the Professional Services and OT/ICS solutions teams directly, since Forescout's Professional Services Engineer roles explicitly cover Zero Trust segmentation, IT/OT convergence, and OT/ICS innovation; also explore federal/government vertical given DISA Comply-to-Connect (C2C) work referenced in job postings.</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>SVP Lifecycle Services; Senior Global Product Manager, Cybersecurity Projects; Director OT Cybersecurity Consulting; NA Sales Director, Industrial Cybersecurity Services</t>
+          <t>VP Professional Services; Director OT/ICS Solutions; Head of Federal/Government Cybersecurity; VP Solutions Engineering; Director Zero Trust Segmentation Practice</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Rockwell Automation SecureOT; Verve Industrial Protection Rockwell; Rockwell Automation OT cybersecurity consultant; Rockwell Automation Lifecycle Services cybersecurity</t>
+          <t>Forescout OT security; Forescout Professional Services Engineer; Forescout Comply to Connect; Forescout IT/OT convergence; Forescout Zero Trust segmentation</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -2183,11 +2175,11 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>Active listings found for OT Cybersecurity Consultant, Senior OT Cybersecurity Consultant, Cybersecurity Services Sales Executive (SecureOT suite), Lead AI Security Architect, and Senior Security Engineer roles across multiple U.S. locations at research time.</t>
+          <t>Glassdoor reports Forescout is currently hiring for 10 open positions in the United States as of June 2026; additional listings found for Professional Services Engineer, Software Engineering Manager, and Strategic Sourcing Specialist roles.</t>
         </is>
       </c>
       <c r="R16" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
@@ -2196,7 +2188,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>https://www.rockwellautomation.com/en-us/capabilities/industrial-cybersecurity/welcome-to-a-new-era-of-ot-security.html</t>
+          <t>https://www.forescout.com/company/careers/</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2210,42 +2202,34 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>LeveL5Cyber</t>
+          <t>Tenable Holdings, Inc.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://www.level5cyber.com/</t>
+          <t>https://www.tenable.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Boutique OT/ICS Cybersecurity Consultancy</t>
+          <t>Cybersecurity Product Vendor (Exposure Management / Vulnerability Management with OT Security line)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>United States (exact city/state not confirmed via search)</t>
+          <t>Columbia, Maryland, USA</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Cross-sector industrial: Oil &amp; Gas, Mining, Chemical/Petrochemical, Energy &amp; Utilities, Life Sciences/Pharma, Food &amp; Beverage, Financial Services, Defense Industrial Base (DIB), Agriculture, Water &amp; Wastewater</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Small (boutique, likely &lt;50 employees) (estimate)</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>$1M-$25M (estimate)</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>estimate</t>
+          <t>Vulnerability/exposure management software provider with a dedicated OT/ICS security product line (Tenable OT Security / Tenable One OT Exposure) serving energy, manufacturing, healthcare, government, and critical infrastructure sectors</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>public-company (see EDGAR)</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -2260,41 +2244,41 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>LeveL5Cyber is a pure-play OT/ICS cybersecurity advisory firm. &lt;cite index="1-3"&gt;Their services include Risk Assessments, OT Network Segmentation Programs, OT Consulting &amp; Enablement, Post-Segmentation Support Services, OT Firewall Lifecycle Management, and Acquisition Integrations, and the company was forged by a group of experienced leaders highly skilled in the protection of critical infrastructure.&lt;/cite&gt; &lt;cite index="7-15"&gt;They follow industry-leading cybersecurity standards for infrastructure businesses: NIST 800 series, CMMC, ISA/IEC 62443, and ISO.&lt;/cite&gt; This is an ideal small-firm target for an OT security consultant seeking a specialist advisory environment.</t>
+          <t>Tenable is a pure-play cybersecurity vendor whose platform explicitly extends into OT: the company markets a 'Secure OT/IoT' solution designed to "bridge the gap between IT and OT to manage security across your entire cyber-physical ecosystem." It is Nasdaq-listed (TENB) and is an SEC filer, so precise financials/headcount should be sourced from EDGAR rather than estimated here.</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Active content marketing and conference presence — &lt;cite index="4-12"&gt;members of their team attended the S4x24 conference in Miami to discuss the latest in OT and ICS&lt;/cite&gt;. Broad and expanding industry vertical coverage (mining, oil &amp; gas, life sciences, financial services, chemical, food, DIB) suggests active business development across sectors.</t>
+          <t>Tenable reported at December 31, 2025, Tenable served over 40,000 customers, including about 65% of the Fortune 500 and about 50% of the Global 2000, and reported backlog of $159.9 million, up from $33.2 million a year earlier. Job boards show active postings referencing OT-specific consulting work with Tenable's platform, e.g. an OT Cybersecurity / Tenable OT Consultant role tied to a municipal utility RFP, indicating expanding OT go-to-market activity.</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Direct outreach to founders/leadership via LinkedIn given small firm size; highlight specific OT segmentation, firewall lifecycle, or risk assessment experience; reference S4x24/ICS community engagement as a conversation starter; consider partnership/subcontractor angle given their apparent boutique consulting model.</t>
+          <t>Target Tenable's OT/ICS product, sales engineering, and customer success organizations directly, and also approach Tenable's channel/reseller/MSSP partners (who deliver OT security services using Tenable's platform) as a services-oriented entry point given the candidate's advisory background.</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Managing Partner/Principal; VP OT Cybersecurity Consulting; Director of Industrial Cybersecurity Services; Practice Lead ICS/OT Security</t>
+          <t>VP/Director OT Security Product; Director Industrial/OT Solutions Engineering; Head of Critical Infrastructure Security; Director Energy &amp; Government Vertical Sales; OT Security Practice Lead (Partner/Channel)</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>LeveL5Cyber; OT cybersecurity consulting boutique; ICS security advisory firm; OT network segmentation consultant</t>
+          <t>Tenable OT; Tenable.ot; Tenable Operational Technology; Tenable Exposure Management OT; Tenable critical infrastructure</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>No specific current job openings found via web search; company website emphasizes services rather than a careers page in search results.</t>
+          <t>Tenable's careers site and third-party job boards (Indeed, ZipRecruiter, LinkedIn) show ongoing openings across sales engineering, security research, and customer-facing roles, plus partner-driven OT consulting demand; the company states Jobs are categorized as Hub (office-based) or Field-based... Field/Remote roles directly engage with customers and partners, indicating active recruiting across functions relevant to OT-facing roles.</t>
         </is>
       </c>
       <c r="R17" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
@@ -2303,7 +2287,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>https://www.level5cyber.com/</t>
+          <t>https://www.tenable.com/careers</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2317,38 +2301,38 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Booz Allen Hamilton</t>
+          <t>Deloitte Risk &amp; Financial Advisory (Deloitte &amp; Touche LLP)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://www.boozallen.com/</t>
+          <t>https://www2.deloitte.com/us/en/pages/risk/solutions/ot-iot-energy-and-chemicals-cybersecurity.html</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Large Systems Integrator / Management &amp; Technology Consulting (Federal + Commercial Cyber)</t>
+          <t>Big 4 Professional Services / Cyber Risk Advisory Practice</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>McLean, Virginia, USA</t>
+          <t>New York, NY, USA (Deloitte US member firm; global network HQ in London, UK)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Federal/Defense (DoD, Intelligence Community), Critical Infrastructure (energy, pharmaceutical, manufacturing, water), Commercial Fortune 500/Global 2000</t>
+          <t>Enterprise cyber risk consulting with a dedicated global OT/ICS cybersecurity practice serving energy, chemicals, manufacturing, life sciences, utilities and other industrial sectors</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Large (Public company, tens of thousands of employees)</t>
+          <t>10,000+ (large multinational professional services firm)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>public-company (see EDGAR)</t>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
@@ -2363,27 +2347,27 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Booz Allen has a dedicated, mature OT/ICS cybersecurity practice spanning federal and commercial markets. &lt;cite index="12-1"&gt;Booz Allen's OT Cybersecurity Lab supports securing industrial control systems (ICS) and OT in critical infrastructure by providing a testing environment for developing and evaluating new capabilities.&lt;/cite&gt; &lt;cite index="12-22,12-23"&gt;Their integrated team of industrial control systems engineers, cybersecurity specialists, and strategists supports customers across critical infrastructure sectors, protecting OT environments, employee safety, and the bottom lines, using a threat-focused approach to help identify vulnerabilities, prioritize remediation, and carry out large-scale OT cybersecurity transformations.&lt;/cite&gt; They also serve &lt;cite index="12-7"&gt;10 of the top 20 global pharmaceutical companies, 3 of the top oil and gas companies, and 3 of the top global automakers&lt;/cite&gt;, and maintain an OT/ICS SOC-as-a-Service offering plus a specific SAF-ICS OT risk assessment lifecycle methodology.</t>
+          <t>Deloitte Risk &amp; Financial Advisory runs one of the largest dedicated OT cybersecurity advisory practices among the Big 4, with named leadership roles such as a US and Global Cyber OT Leader for Deloitte Risk &amp; Financial Advisory and a global delivery team described as a core worldwide team of 1,500+ OT cybersecurity specialists in key operational and manufacturing regions worldwide. Deloitte has also made inorganic investments in this space, having announced today its acquisition of the industrial cybersecurity business (aeCyberSolutions) from Greenville, S.C.-based Applied Engineering Solutions, Inc. (aeSolutions) to bolster ICS/OT frameworks and tooling, and maintains a technology alliance in which Deloitte's Cyber Risk Services end-to-end Industrial Control Systems (ICS) Security offering, enabled by the Dragos platform, helps organizations manage their cyber risks in the ICS and Operational Technology (OT) environments.</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>&lt;cite index="18-9"&gt;Today, the company has over 8,000 cyber professionals delivering on nearly 300 active cyber projects ranging from small, innovative task orders to marquee&lt;/cite&gt; engagements. &lt;cite index="18-5,18-6"&gt;Booz Allen Hamilton was named top federal cybersecurity provider, projecting $2.8 billion in cyber revenue by FY25, leading in cyber-related prime contract obligations from the federal government in fiscal years 2021 to 2023 per Deltek's GovWin analysis.&lt;/cite&gt; Actively posting OT/ICS-specific analyst and consultant roles on their careers site and LinkedIn.</t>
+          <t>Deloitte continues to expand and market OT-specific service lines such as Factory Accelerated Security Transformation (FAST) and a Managed XDR offering for OT, and actively recruits OT/ICS specialists; job postings include a dedicated Cyber Operational Technology/ Industrial Control Systems (OT/ICS) Senior Consultant role recruiting through the end of 2026, requiring hands-on experience with Claroty, CrowdStrike-for-OT, BeyondTrust and other ICS security tools.</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Target through federal/commercial OT cybersecurity practice leads; leverage their published thought-leadership (Industrial Cyber contributor articles) as talking points; approach via LinkedIn recruiters posting OT/ICS roles or via their Commercial Solutions / Civil Government business units.</t>
+          <t>Approach via Deloitte's Cyber &amp; Strategic Risk / OT Cybersecurity service line leadership and industry sector teams (Energy &amp; Chemicals, Manufacturing, Power &amp; Utilities), referencing specific practice offerings (Cyber PHA, FAST, MXDR-OT) to align candidate's OT advisory background with named engagement types.</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>VP Cyber-Physical Defense; Director OT/ICS Cybersecurity; Principal OT Cybersecurity Consultant; Senior Lead OT Cybersecurity Practice</t>
+          <t>Principal/Managing Director, Cyber OT Practice; US/Global Cyber OT Leader; Cyber IoT Leader; OT/ICS Cybersecurity Architect (Senior Consultant/Manager); Cyber Risk Services - Energy &amp; Chemicals Industry Leader</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Booz Allen OT/ICS Cybersecurity; Booz Allen cyber-physical defense; Booz Allen SAF-ICS; Booz Allen industrial control systems consultant</t>
+          <t>Deloitte Cyber OT; Deloitte ICS/OT cybersecurity; Deloitte Risk &amp; Financial Advisory OT; Deloitte aeCyberSolutions; Deloitte Cyber-Physical Systems</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -2393,7 +2377,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>&lt;cite index="16-1,16-8"&gt;Active LinkedIn/careers postings for an OT/ICS Cybersecurity Analyst role supporting DoD and Federal Agency client projects within the Cybersecurity domain, consulting with clients on secure design of OT and ICS environments.&lt;/cite&gt;</t>
+          <t>Deloitte has an active, dedicated posting for a Cyber OT/ICS Senior Consultant (recruiting through 12/31/2026) plus numerous broader Cyber Risk Services openings on its own careers portal and third-party boards, indicating ongoing OT-specific recruitment.</t>
         </is>
       </c>
       <c r="R18" t="n">
@@ -2406,7 +2390,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>https://www.boozallen.com/markets/commercial-solutions/operational-technology-ot-cybersecurity-for-business.html</t>
+          <t>https://www.deloitte.com/global/en/services/consulting/services/cyber/deloittes-operational-technology-cybersecurity-services.html</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2420,38 +2404,42 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Wood plc (Wood Group / John Wood Group)</t>
+          <t>Wood plc (John Wood Group, North America)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://www.woodgroup.com/</t>
+          <t>https://www.woodgroup.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Global Engineering, Automation &amp; Systems Integration Consultancy</t>
+          <t>Engineering, Consulting &amp; Project Delivery Firm (with OT Cybersecurity service line)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Aberdeen, Scotland, UK</t>
+          <t>Aberdeen, Scotland, UK (major North America hub: Houston, TX)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Oil &amp; Gas (Upstream, Midstream, Petrochemicals &amp; Refining), Life Sciences/Pharma, Chemicals, Minerals &amp; Metals, Power, Renewables, Carbon Capture, Hydrogen</t>
+          <t>Energy, oil &amp; gas, chemicals, power, renewables, mining and industrial engineering/consulting, with a dedicated OT/control-systems cybersecurity consulting offering</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Large (Public company, global engineering firm)</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>public-company (see EDGAR)</t>
+          <t>~25,000-55,000 employees globally (varies by source/date)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>$4B-$6B (estimate; group historically reported multi-billion dollar revenue; company recently went private)</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>estimate</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -2466,45 +2454,45 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Wood has an established, long-running Industrial OT Cybersecurity practice integrated with its automation/controls engineering business, distinguishing it from pure-play cyber firms. &lt;cite index="21-16,21-17"&gt;Wood combines OT cybersecurity expertise with decades of experience in automation, control systems and systems integration, with specialists who understand how industrial environments operate and help organisations identify vulnerabilities, assess risk and implement practical security improvements tailored to their operational requirements.&lt;/cite&gt; &lt;cite index="23-3,23-4"&gt;They market OT cybersecurity consulting with 25+ years experience, 500+ specialists, and 200+ clients.&lt;/cite&gt; Their broader automation &amp; controls business is sizable: &lt;cite index="22-3"&gt;Wood's automation and control solutions are provided globally by around 1,400 dedicated technical staff across a network of 41 offices in 17 countries.&lt;/cite&gt;</t>
+          <t>Wood explicitly markets an OT cybersecurity consulting practice, stating it offers to Protect your OT systems with expert cybersecurity consulting. 25+ years experience, 500+ specialists, 200+ clients, combining this with its deep legacy in automation, control systems and systems integration... help organisations identify vulnerabilities, assess risk and implement practical security improvements tailored to their operational requirements. However, note a major corporate change: Wood is was acquired by Sidara Limited, an entity controlled by Dar-Al Handasah Consultants Shair and Partners Holdings Limited ("Sidara"), and its shares were delisted from the London Stock Exchange in March 2026, following a period of serious financial and governance distress, so it is no longer a standalone public filer.</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>&lt;cite index="21-18"&gt;With manufacturing remaining the most targeted industry for cyberattacks and ransomware activity continuing to increase across industrial sectors, effective OT security has become a key part of operational resilience&lt;/cite&gt; — a narrative Wood is actively using in its marketing, alongside statistics like &lt;cite index="21-28"&gt;about 1 in 4 operators had to shut down due to OT security incidents last year&lt;/cite&gt;. Actively recruiting for a dedicated Industrial Cybersecurity Consultant role focused on North America growth.</t>
+          <t>Post-acquisition, Wood is described as retaining its own brand: Wood will retain its own brand and continue operating as a standalone business, while benefiting from Sidara's global scale and long-term owner-operator mindset, and the combined Sidara-Wood group now generates more than 55,000 professionals... over $8.5bn in revenue across all geographies, with approximately 40 percent in North America. This suggests renewed financial stability and potential investment capacity for service lines like OT cybersecurity, though the parent deal followed a period where there was a c.80% fall in its share price, its shares were suspended and the FCA launched an investigation, and Wood also disclosed a late-2025 data breach... affecting one of the United Kingdom's largest engineering and consulting firms, which may itself create urgency around cyber resilience investment.</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Approach via Wood's Digital Integration / Automation &amp; Systems Integration business unit leadership; reference their ISA/IEC 62443 and NIST CSF-aligned Asset Protection Solutions practice; target North America energy/materials growth initiatives given active hiring signal in Houston, TX.</t>
+          <t>Engage through Wood's Consulting business unit and its dedicated cybersecurity-for-OT service page/team, emphasizing the candidate's ability to support post-acquisition stabilization and growth of the OT security consulting practice under new Sidara ownership; North America entry point likely via the Houston energy/oil &amp; gas hub.</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Business Manager Digital Integration; Director Industrial Cybersecurity; VP Automation &amp; Control / OT Security; Principal ICS Cybersecurity Consultant</t>
+          <t>Director/Head of OT Cybersecurity Consulting; VP Digital Consulting - Energy &amp; Industrial; Director Automation &amp; Control Systems Security; Consulting Practice Lead - Cybersecurity; Executive President, Consulting &amp; Projects (org context)</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Wood plc OT cybersecurity; Wood Group industrial cybersecurity consultant; Wood Digital Integration ICS; John Wood Group cybersecurity</t>
+          <t>Wood plc OT cybersecurity; Wood Group ICS security; Wood consulting cybersecurity control systems; Wood plc digital consulting; Wood Sidara cybersecurity</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>&lt;cite index="32-1,32-3,32-4"&gt;Actively hiring an Industrial Cybersecurity Consultant in Houston, TX, accountable for Wood's Industrial Cybersecurity and Digital Integration business growth and delivery across Energy and Materials industries in North America, providing principal consulting on ICS Cybersecurity to customers and project teams.&lt;/cite&gt;</t>
+          <t>General hiring activity is high across engineering, technical and trades roles (e.g., 150+ open jobs per Indeed, 485+ per LinkedIn in the US), but no specific current job postings for OT-cybersecurity consulting roles were found in this search; the recent Sidara acquisition and prior restructuring create some uncertainty about near-term hiring pace for the cybersecurity practice specifically.</t>
         </is>
       </c>
       <c r="R19" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>AI research (verify)</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
@@ -2523,44 +2511,98 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Wood plc (Wood Group)</t>
+          <t>NCC Group Security Services, Inc.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://www.woodgroup.com</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
+          <t>https://www.nccgroup.com</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Global Cybersecurity Consulting &amp; Managed Services Firm (OT/ICS Practice)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Manchester, UK (global HQ); US entity operates across 35+ global offices</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Cross-sector: energy &amp; utilities, manufacturing, transport/rail, maritime, automotive, critical national infrastructure</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2,000+ employees globally (per company statements)</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>This company wasn't included in the enrichment response — found via research but details weren't populated. Re-run to try again.</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
+          <t>NCC Group runs a dedicated OT/ICS cybersecurity practice offering Facility Due Diligence risk assessments, safety case analysis (via its Adelard team), and IEC 62443-aligned consulting for industrial clients. Its Energy &amp; Utilities Practice explicitly addresses ICS/OT environments, and the firm recently expanded its OT incident response capability through a partnership with Dragos, combining NCC's DFIR and OT expertise with Dragos's industrial cybersecurity platform for end-to-end IT/OT breach response. NCC Group also holds NCSC CHECK/CIR accreditations and was named a strong performer in Forrester's Cybersecurity Consulting Services Wave.</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>In November 2025, NCC Group announced an enhanced partnership with Dragos to launch a combined IT/OT convergence incident response retainer service, and its DFIR capability was recently recognized in the IDC MarketScape as a 'Major Player.' The firm's strategic roadmap explicitly targets deeper Cloud and OT security capability expansion alongside US market growth.</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Target the Energy &amp; Utilities and Industrials practice leadership; reference the Dragos partnership and Facility Due Diligence service line as points of alignment; approach via LinkedIn posts from the Director of Industrials and Global Head of Threat Intelligence.</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Director of Industrials; VP/Head of Operational Technology Security; Practice Lead - Critical National Infrastructure; Director Facility Due Diligence</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>NCC Group OT security; NCC Group Facility Due Diligence; NCC Group Industrials practice; NCC Group Dragos partnership; NCC Group ICS/SCADA</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Active listings observed on Built In, Glassdoor, and LinkedIn for security engineering, SOC, detection engineering, and cyber consulting roles; no OT-specific req identified at time of research, but hiring activity is ongoing across cyber security functions.</t>
+        </is>
+      </c>
+      <c r="R20" t="n">
+        <v>8</v>
+      </c>
       <c r="S20" t="inlineStr">
         <is>
           <t>AI research (verify)</t>
         </is>
       </c>
-      <c r="T20" t="inlineStr"/>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>https://www.nccgroup.com/consulting-implementation/operational-technology/</t>
+        </is>
+      </c>
       <c r="U20" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2572,38 +2614,38 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>DNV Cyber</t>
+          <t>Parsons Corporation</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.dnv.com/cyber/</t>
+          <t>https://www.parsons.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>OT/IT Cybersecurity Consulting &amp; Advisory (part of global TIC/assurance group)</t>
+          <t>Global Engineering, Defense &amp; Critical Infrastructure Prime Contractor with OT/ICS Cyber Practice</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Høvik, Norway (DNV Group); DNV Cyber operational hubs in Norway, Finland, Sweden, Denmark, Netherlands, Germany</t>
+          <t>Centreville, Virginia, USA</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Maritime, energy (oil &amp; gas, power, renewables), critical infrastructure, healthcare, manufacturing</t>
+          <t>Defense, intelligence, and critical infrastructure: energy grids, water treatment, pipelines, transportation, rail, telecom towers</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>500+ (DNV Cyber division); DNV Group overall is much larger (tens of thousands)</t>
+          <t>18,000+ employees (per company careers materials)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>public-company (see EDGAR)</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -2618,27 +2660,27 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>DNV Cyber is a dedicated IT/OT cybersecurity services arm formed from the 2024 merger of Nixu, Applied Risk, and DNV's own cyber unit, explicitly focused on securing critical infrastructure. Their global team of more than 500 experts brings over 30 years of IT and OT security experience, and they offer OT-specific services including penetration testing, risk assessments, and IEC 62443-aligned assessments.</t>
+          <t>Parsons has decades of experience designing, building, and protecting critical infrastructure and has developed converged OT/IT offerings such as Domain6 (described as the first fully converged solution to thwart attacks on operational technology and information technology environments) and Cyberzcape Tracker, a holistic cyber solution combining passive monitoring with active threat neutralization for critical infrastructure networks, built partly from its acquisition of IPKeys Cyber Partners. The company states it has significant critical infrastructure, industrial control system, and SCADA experience.</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>DNV recently acquired CyberOwl to strengthen maritime cybersecurity, and DNV Cyber has significant ambitions to rapidly grow its Cyber Security unit in the coming years, building on strengths in the Nordics for global impact.</t>
+          <t>Parsons acquired IPKeys Power Partners in 2023 to bolster critical infrastructure cyber offerings, launched the Cyberzcape Tracker product, and continues to publish OT/ICS thought leadership (e.g., an August 2025 piece urging ICS/OT-specific tabletop exercises). The company is actively recruiting for IT/OT/Cyber Security Engineer roles on large infrastructure programs (e.g., rail projects).</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Target via DNV's dedicated careers portal (jobs.dnv.com and careers.nixu.com) and LinkedIn; engage with DNV Cyber's energy/maritime industry leads and highlight IEC 62443 / NIS2 compliance expertise given DNV's strong regulatory advisory angle.</t>
+          <t>Engage through Parsons' Federal Solutions / Critical Infrastructure Protection business unit and its Sealing Technologies cybersecurity subsidiary; reference Domain6/Cyberzcape and IPKeys integration work as conversation starters; monitor Parsons' careers site and Workday postings for OT-specific reqs.</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Head of Sales Industrial &amp; OT Cybersecurity; Head of Cyber Security Maritime; VP OT/ICS Security Services; Director Industrial Cybersecurity</t>
+          <t>VP Cybersecurity - Critical Infrastructure; Director OT/ICS Security; Chief Technology Officer - Critical Infrastructure Protection; Director Cyber &amp; Intelligence Solutions</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>DNV Cyber OT security; DNV Cyber industrial control systems; DNV Cyber IEC 62443; Nixu Applied Risk DNV cyber; DNV maritime cybersecurity</t>
+          <t>Parsons Corporation OT cybersecurity; Parsons ICS SCADA; Parsons critical infrastructure protection; Parsons Domain6; Parsons Cyberzcape; Parsons IPKeys</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -2648,7 +2690,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>DNV maintains active job postings for OT/cyber security consultants across multiple regions (e.g., Singapore Senior OT Cyber Security Consultant listing, DNV Maritime Cyber Security Control System Engineer roles), and DNV Cyber has significant ambitions to rapidly grow its Cyber Security unit in the coming years.</t>
+          <t>A live posting for 'Senior IT/OT/Cyber Security Engineer' on a large-scale rail infrastructure project was found on Parsons' careers site, and Glassdoor lists dozens of open cybersecurity-related roles across Parsons.</t>
         </is>
       </c>
       <c r="R21" t="n">
@@ -2661,7 +2703,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>https://www.dnv.com/cyber/about/our-story/</t>
+          <t>https://www.parsons.com/securing-critical-infrastructure/</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2675,38 +2717,42 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Kudelski Security</t>
+          <t>GRIMM (GRIMM Cyber R&amp;D / SMFS Inc.)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://kudelskisecurity.com/</t>
+          <t>https://grimmcyber.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Cybersecurity consulting/MDR/advisory (division of publicly listed Kudelski Group)</t>
+          <t>Boutique Cyber-Physical (CyPhy)/OT-ICS Security Research &amp; Consulting Firm</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Cheseaux-sur-Lausanne, Switzerland (2nd HQ Phoenix, Arizona, USA)</t>
+          <t>Arlington, Virginia, USA (with a research lab location in Sparta/Cedar Springs, Michigan)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Manufacturing, critical infrastructure, industrial/cyber-physical systems, enterprise &amp; public sector</t>
+          <t>Industrial control systems (ICS), automotive, aerospace/defense, advanced manufacturing, energy, embedded/IoT systems, smart city</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Parent Kudelski Group ~1,600-1,850 employees; Kudelski Security is a division, exact headcount not separately disclosed</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>public-company (see EDGAR/SIX filings - Kudelski SA trades on SIX Swiss Exchange, ticker KUD)</t>
+          <t>11-50 employees (estimate)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>$5M-$25M (estimate)</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>estimate</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
@@ -2721,27 +2767,27 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Kudelski Security offers a purpose-built MDR for OT, providing 24×7 detection, analysis, and response to threats within OT systems like PLCs, SCADA, and sensor networks. Its Cyber Fusion Centers integrate Claroty industrial cybersecurity technology, and the company also lists dedicated OT Security Assessment and CPS Security Assessment advisory offerings, plus a Third-Party Risk Management (OT) service.</t>
+          <t>GRIMM specializes in CyPhy security engineering combining hardware, firmware, and software expertise, with explicit ICS/OT capabilities including its ICS Wall demonstrating vulnerabilities in power and energy OT environments. GRIMM's SVP leads a dedicated CyPhy Product group focused on securing industrial control systems, and GRIMM co-founded the nonprofit ICS Village used at S4x and BSides events. The firm recently partnered with TXOne Networks to deliver a full suite of OT cybersecurity offerings for manufacturing and critical infrastructure/ICS clients.</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Kudelski Security has been recognized 3x as a Leading Provider in the Forrester Wave for Managed Detection and Response (2021-2025) and 6x as a Representative Vendor in Gartner's Market Guide for Digital Forensics and Incident Response Retainer Services, indicating sustained analyst-recognized growth in its MDR/OT security line.</t>
+          <t>New strategic partnership announced with TXOne Networks for OT security tooling (Stellar, Edge, Portable Inspector), continued presence at S4x and ICS Village events, and repeated Inc. 5000 honoree status across multiple years, indicating sustained revenue growth.</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Engage through Kudelski Security's OT &amp; CPS practice pages and LinkedIn; target the OT/CPS security management and advisory groups; leverage Kudelski's Claroty partnership and Cyber Fusion Center staffing needs as an entry point for OT-focused advisory roles.</t>
+          <t>Engage directly with the CyPhy Product group leadership and CEO via LinkedIn; leverage community touchpoints like ICS Village, S4x conferences, and GRIMMCon; highlight alignment with automotive/ICS/embedded security niche.</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Director OT &amp; CPS Security; VP Managed Detection and Response; Head of Industrial Cybersecurity Advisory; Practice Lead OT Security Assessment</t>
+          <t>SVP/VP CyPhy Product Group; Director OT/ICS Security Practice; Head of Industrial Cybersecurity Consulting</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Kudelski Security OT; Kudelski Security MDR industrial; Kudelski Cyber Fusion Center OT; Kudelski Security CPS; Kudelski Security Claroty</t>
+          <t>GRIMM Cyber OT security; GRIMM CyPhy; GRIMM ICS Village; SMFS Inc GRIMM cybersecurity; GRIMM TXOne Networks partnership</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -2751,11 +2797,11 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>No specific current OT/cyber job postings were surfaced in this search; company site emphasizes active MDR/OT service offerings but explicit open requisitions were not confirmed at research time.</t>
+          <t>GRIMM maintains an active careers page inviting applicants and interns, but no specific current OT/ICS job requisitions were identified in search results at time of research.</t>
         </is>
       </c>
       <c r="R22" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S22" t="inlineStr">
         <is>
@@ -2764,7 +2810,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>https://kudelskisecurity.com/solutions/by-need/secure-ot-ics-networks/</t>
+          <t>https://grimmcyber.com/who-we-are/</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2778,37 +2824,37 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>exida, LLC</t>
+          <t>Applied Control Solutions, LLC</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://www.exida.com/</t>
+          <t>https://www.appliedcontrolsol.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Functional Safety &amp; IACS Cybersecurity Consulting/Certification</t>
+          <t>Boutique OT/ICS Cybersecurity Consulting &amp; Advisory</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Sellersville, Pennsylvania, USA (also offices in Germany, Canada, Mexico, UK, Ireland, UAE, South Africa, Italy)</t>
+          <t>Cupertino, California, USA</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Process industry (chemical, oil &amp; gas), automotive, machinery, energy, pharmaceuticals, medical devices, railway</t>
+          <t>Industrial control systems (ICS) cybersecurity across critical infrastructure sectors (electric power, oil &amp; gas, water, manufacturing, maritime); specific focus on Level 0/1 field device and process sensor cybersecurity</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>51-200 employees (estimate; some sources report ~100-250)</t>
+          <t>Micro (likely 1-10 employees / solo-practitioner-led firm)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>$10M-$30M (estimate)</t>
+          <t>&lt;$5M (estimate)</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -2828,41 +2874,41 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>exida is an industrial control system (ICS) and SCADA system security consulting and certification firm that focuses on the unique requirements of industrial automation and process control systems based on the ISA/IEC-62443 standard. The firm combines deep functional safety expertise (IEC 61508/61511) with IACS cybersecurity consulting, assessment, and certification services, serving Fortune 500 to small companies across chemical, oil &amp; gas, power, and automotive sectors.</t>
+          <t>This is essentially the firm of Joe Weiss, a foundational figure in OT/ICS cybersecurity. Per company materials, &lt;cite index="42-1,42-2"&gt;Joe Weiss of Applied Control Solutions helped start control system (now OT) cyber security in 2000, coming from a background in instrumentation, control, and safety systems melded with cyber security expertise&lt;/cite&gt;. The firm's differentiator is a unique incident dataset: &lt;cite index="42-5,42-6"&gt;Weiss has amassed a non-public database of more than 11 million control system cyber incidents, and his knowledge allows him to provide expert consulting to governments, end-users, equipment suppliers, and cyber security companies&lt;/cite&gt;. The current site describes the firm's focus as &lt;cite index="44-1"&gt;helping critical-infrastructure operators recognize control system automation incidents that put people and operations at risk — through on-site workshops, an annual incident service, and trusted sharing&lt;/cite&gt;.</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>exida continues to expand its cybersecurity training and certification offerings (e.g., exSILentia Cyber software updates for IEC 62443-3-2 risk assessments) and hosts recurring international symposiums on functional safety and cybersecurity, suggesting steady niche-market growth rather than rapid scaling.</t>
+          <t>No evidence of headcount growth or funding events; this appears to be a stable, small consulting practice rather than a scaling company. A recent (2026-dated) site refresh at appliedcontrolsol.com suggests some renewed marketing/branding activity, but no hiring or expansion signals were found.</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Approach via exida's direct careers/consulting contact channels and LinkedIn given its small, specialized consultant base; target functional safety + cybersecurity dual-expertise practitioners; leverage exida's IEC 62443/IEC 61508 certification body reputation as a talking point for OT advisory engagements.</t>
+          <t>Approach as a potential referral partner, subcontractor, or alliance for large-account OT assessments (rather than a direct employer with open headcount) — this is a niche, expert-led boutique; best fit is proposing collaboration on assessments, Level 0/1 sensor security engagements, or co-authored thought leadership/incident-sharing initiatives rather than applying to a formal job posting.</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Director IACS Cybersecurity; VP Functional Safety &amp; Cybersecurity Services; Principal Consultant OT Security; Practice Lead ISA/IEC 62443</t>
+          <t>Managing Partner; Principal Consultant OT/ICS Security; Director of Control System Cybersecurity</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>exida IACS cybersecurity; exida IEC 62443; exida functional safety consultant; exida OT security; exida CFSE</t>
+          <t>Applied Control Solutions LLC; Joe Weiss ICS cybersecurity; Level 0 process sensor cybersecurity; control system cyber incident database</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>No</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>Third-party data (ZoomInfo) referenced an office move affecting about 12 employees, but no specific current open OT/cyber roles were confirmed via this search; company size suggests infrequent but specialized hiring.</t>
+          <t>No job postings, careers page, or hiring signals were found; the firm's web presence (realtimeacs.com) shows a placeholder 'coming soon' site, and the primary site (appliedcontrolsol.com) is consultant-bio focused with no listed openings.</t>
         </is>
       </c>
       <c r="R23" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="S23" t="inlineStr">
         <is>
@@ -2871,7 +2917,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>https://www.exida.com/ICS-Cybersecurity/Resources</t>
+          <t>https://www.appliedcontrolsol.com/about</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2885,37 +2931,37 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Armexa</t>
+          <t>Xage Security, Inc.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://armexa.com/</t>
+          <t>https://xage.com</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>OT/ICS Cybersecurity Consulting &amp; Services Boutique</t>
+          <t>OT/IT/Cloud Zero Trust Cybersecurity Vendor (Software/Platform)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Palo Alto, California, USA</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Oil &amp; gas, LNG, chemicals, pipelines, power/utilities, manufacturing, building automation, healthcare</t>
+          <t>Zero trust identity, access management, and remote access for critical infrastructure sectors including energy/oil &amp; gas, utilities, defense/space, manufacturing, and logistics</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>~30-50 employees (estimate)</t>
+          <t>~100-115 employees</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>$5M-$25M (estimate)</t>
+          <t>$10M-$50M (estimate)</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -2935,37 +2981,37 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Armexa is a boutique, pure-play industrial cybersecurity firm. &lt;cite index="2-11"&gt;Established in 2021 and headquartered in Houston, with 30+ OT cybersecurity engineers and consultants, industry-recognized leaders with a rich history of expertise in industrial IT/OT and cybersecurity.&lt;/cite&gt; &lt;cite index="2-12,2-13"&gt;The firm provides full-spectrum OT security services, from governance and program development to system design, implementation &amp; ongoing support, with decades of hands-on experience in critical infrastructure facilities such as chemical plants, refineries, pipelines, manufacturing, and offshore facilities.&lt;/cite&gt; It's a strong target for an OT security consulting/advisory job seeker given its asset-owner-mentality consulting model.</t>
+          <t>Xage is a venture-backed pure-play OT/IT zero trust security vendor. Per Tracxn, &lt;cite index="11-16,11-17"&gt;Xage Security is a series B company based in Palo Alto, founded in 2016 by Kamesh Raghavendra and Susanto Irwan, operating as a provider of a blockchain based security platform for IoT applications&lt;/cite&gt;, and &lt;cite index="11-18"&gt;has raised $80M in funding from investors like Chevron, SAIC and Aramco Ventures&lt;/cite&gt;. Its positioning per its own site: &lt;cite index="39-13,39-14"&gt;Xage provides zero trust access control across any type of asset, anywhere in the enterprise across IT, OT, and cloud, enforcing granular protection without coming at the expense of agility or usability&lt;/cite&gt;. Notably, per ZoomInfo, &lt;cite index="18-27,18-28"&gt;Xage has integrated with NVIDIA DOCA security and NVIDIA BlueField to deliver line-speed policy enforcement for AI factory scale, and reports 81% revenue growth driven by a global shift from perimeter-based tools to identity-driven protection for AI infrastructure and critical systems&lt;/cite&gt;, indicating strong recent momentum.</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Recently expanded via a formal channel/services partnership: &lt;cite index="10-1,10-2"&gt;Global automation company Emerson and Armexa announced a strategic collaboration to offer customers using Emerson's DeltaV automation platform, a global suite of advanced OT cybersecurity services, giving DeltaV customers a single, authorized cybersecurity services provider.&lt;/cite&gt; The firm also touts deep penetration into the LNG sector: &lt;cite index="8-2"&gt;Armexa's team has secured OT environments at 5 of the 9 US LNG export terminal complexes that collectively represent over 80% of America's operational LNG export capacity, and every LNG operator Armexa has worked with has returned for additional engagements.&lt;/cite&gt;</t>
+          <t>Strong recent growth signals: 81% reported revenue growth and new NVIDIA-integrated AI security products (per ZoomInfo/company announcements); continued VC funding from strategic energy/defense investors (Chevron, SAIC, Aramco Ventures, PETRONAS Ventures per PitchBook); expanding customer testimonials from Kinder Morgan and U.S. Space Force; recent Fortress Cybersecurity Award recognition in 2025.</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Approach via warm intro referencing the Emerson/DeltaV and TXOne partnerships and LNG/pipeline TSA compliance practice; position around specific verticals (LNG, midstream oil &amp; gas, chemicals) where Armexa has public case studies. Small firm — direct outreach to leadership team likely most effective.</t>
+          <t>Target via LinkedIn outreach to sales engineering, solutions advisory, and partnerships leadership; given its enterprise energy/defense customer base (Kinder Morgan, Space Force), position expertise in OT security frameworks (IEC 62443, NERC CIP) as valuable to their solutions advisory and customer success teams; also consider channel/partner angle since Xage sells through system integrators.</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>VP OT Cybersecurity Services; Director Industrial Cybersecurity; Principal Consultant OT/ICS Security; Practice Lead OT Security</t>
+          <t>VP Solutions Engineering; Director OT/Industrial Security; Head of Customer Success - Critical Infrastructure; Director of Partnerships</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Armexa OT cybersecurity; Armexa Houston industrial cyber; Armexa ICS consultant; Armexa CyberHAZOP</t>
+          <t>Xage Security; Xage Fabric zero trust; Xage OT IT cloud security; Xage Security Palo Alto</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>Armexa maintains an active careers page inviting applications across cybersecurity, engineering, and OT/ICS disciplines, but no specific current open-role count was found via search.</t>
+          <t>Multiple job boards (ZipRecruiter, Indeed, Glassdoor, LinkedIn, Built In) show active open roles, including software engineering, backend engineering, and senior director of partnerships/business development positions as of 2026.</t>
         </is>
       </c>
       <c r="R24" t="n">
@@ -2978,7 +3024,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>https://armexa.com/about-us/</t>
+          <t>https://xage.com/careers/</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -2992,42 +3038,42 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>GRIMM Cyber (SMFS, Inc.)</t>
+          <t>DNV (DNV Cyber / DNV Energy Systems, USA)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://grimmcyber.com/</t>
+          <t>https://www.dnv.com/cyber/</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Cybersecurity R&amp;D / OT-ICS-Embedded Security Consultancy</t>
+          <t>Global Assurance &amp; Risk Management Provider with Dedicated OT/IT Cybersecurity Services Division</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Arlington/Stafford County, VA (also operates a CyPhy R&amp;D lab/facility in Cedar Springs, MI)</t>
+          <t>Oslo, Norway (global HQ); DNV Cyber operates from hubs in Norway, Finland, Sweden, Denmark, Netherlands, Germany, Romania; DNV Energy Systems has significant US presence</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Defense/DoD, automotive, aerospace, manufacturing, energy, critical infrastructure, embedded/IoT systems</t>
+          <t>IT and industrial control system (OT) security across energy, maritime, manufacturing, and other critical infrastructure sectors, including IEC 62443-based OT risk assessment, penetration testing, and managed detection &amp; response (MXDR)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>~11-50 employees (estimate)</t>
+          <t>500+ (DNV Cyber division); DNV Group overall is a large multinational (10,000+ employees)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>~$3M-$10M (estimate)</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>estimate</t>
+          <t>Unknown precise figure (DNV is a Norwegian foundation-owned company, not SEC-registered; large multinational scale)</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -3042,41 +3088,41 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>GRIMM (legal entity SMFS, Inc.) is a specialized cyber-physical/OT security research and consulting firm. &lt;cite index="12-1,12-3,12-4,12-5"&gt;GRIMM is an advanced cybersecurity and mission engineering company specializing in Industrial Control Systems (ICS), Operational Technology (OT), embedded platforms, offensive security, and high-consequence mission systems, helping government and commercial customers identify vulnerabilities, strengthen resilience, and develop strategic advantage, combining hands-on engineering expertise with real-world understanding to solve problems where traditional IT security firms fall short.&lt;/cite&gt; Its heavy involvement in ICS Village and vulnerability research on control systems makes it a strong niche fit for an OT cyber advisory job seeker.</t>
+          <t>DNV Cyber is one of the largest dedicated OT/IT cybersecurity services arms in Europe, built through major acquisitions. As reported, &lt;cite index="51-2,51-3"&gt;DNV created one of Europe's fastest growing cyber security services businesses by merging its existing cyber security business with two recently acquired companies – Nixu and Applied Risk – bringing together more than 500 cyber security experts to safeguard demanding IT and industrial control system environments across multiple industries&lt;/cite&gt;, following &lt;cite index="51-1"&gt;DNV's acquisition of Amsterdam-based industrial cyber security specialist Applied Risk in 2021, and the conclusion of DNV's acquisition of Helsinki-headquartered cyber security services leader Nixu in December 2023&lt;/cite&gt;. Its OT specialization is explicit: &lt;cite index="21-13"&gt;DNV Cyber has expertise and experience covering all the aspects of OT security, including OT/IT convergence&lt;/cite&gt;, and its penetration testing arm notes &lt;cite index="30-2,30-3"&gt;DNV Cyber is driven to safeguard the critical infrastructure our society depends on, combining cyber security knowledge and experience in operational technology to assist asset owners, system integrators and suppliers to develop, deploy and maintain cyber-resilient operations&lt;/cite&gt;.</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>GRIMM has been expanding OT-focused partnerships: &lt;cite index="13-9,13-10"&gt;GRIMM Cyber and TXOne Networks announced a partnership uniting GRIMM's cybersecurity expertise with TXOne's OT security solutions, chosen under the guidance of a Senior VP with 32 years in the field for TXOne's ability to simplify OT security while minimizing downtime.&lt;/cite&gt; It also announced physical footprint growth: &lt;cite index="40-2,40-6"&gt;GRIMM announced plans to invest $435,000 to open a new headquarters location in Stafford County, VA, and to hire approximately 23 new employees following completion of its new corporate headquarters.&lt;/cite&gt;</t>
+          <t>Very strong M&amp;A-driven growth: recent acquisition of CyberOwl to expand into maritime OT security (per Industrial Cyber, 2026); continued publication of regional threat/resilience reports (Denmark, Norway, Sweden, Finland) and monthly threat insights; Microsoft-verified MXDR status recently achieved; DNV was also recently selected for rail cybersecurity work in the Dominican Republic — indicating active market expansion beyond its traditional maritime/energy base.</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Target via its OT/ICS and automotive/embedded practice leads; reference GRIMM's ICS Village and TXOne partnership as talking points. Given small headcount, direct outreach to practice leadership (SVP-level) rather than HR is likely more effective.</t>
+          <t>Target DNV Cyber's OT security consulting practice (former Applied Risk team) directly, as well as DNV Energy Systems USA for North American energy-sector engagements; leverage the recent CyberOwl and rail-sector wins as conversation starters about expanding OT verticals; approach through LinkedIn to practice leads in OT security consulting, penetration testing, and MXDR delivery given the company's stated 11-country footprint and ongoing expert-team growth narrative.</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>SVP CyPhy/OT Security; Director ICS Vulnerability Research; Principal OT/Embedded Security Consultant; VP Government/Commercial Cyber Services</t>
+          <t>Head of OT Security Practice; Director Industrial Cyber Security Consulting; VP Energy Systems Cybersecurity (Americas); Principal OT Security Consultant</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>GRIMM Cyber OT; GRIMM SMFS ICS; GRIMM CyPhy security; GRIMM Cyber vulnerability research</t>
+          <t>DNV Cyber; DNV Applied Risk OT security; DNV Energy Systems cybersecurity; DNV Nixu cyber security; DNV Cyber OT penetration testing</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>GRIMM's own site states an active hiring posture: &lt;cite index="20-7,20-8"&gt;"We are hiring! See our Careers Page for open positions."&lt;/cite&gt; though internship program was noted closed as of a 2024 snapshot.</t>
+          <t>No specific current job postings were retrieved in this search, but given DNV Cyber's stated growth trajectory (500+ experts, multiple recent acquisitions including CyberOwl), continued hiring in OT/cyber consulting roles is highly likely; recommend checking dnv.com/careers directly for current openings.</t>
         </is>
       </c>
       <c r="R25" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S25" t="inlineStr">
         <is>
@@ -3085,7 +3131,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>https://grimmcyber.com/careers/</t>
+          <t>https://www.dnv.com/news/2024/dnv-creates-european-cyber-security-services-powerhouse-through-merger-with-nixu-and-applied-risk/</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3099,35 +3145,39 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Fortress Information Security</t>
+          <t>ITEGRITI Corporation</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.fortressinfosec.com/</t>
+          <t>https://itegriti.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Cyber Supply Chain Risk Management (C-SCRM) / TPRM Platform &amp; Services</t>
+          <t>Boutique OT/IT Cybersecurity &amp; Compliance Advisory Firm</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Orlando, FL</t>
+          <t>Houston, Texas, USA (also lists Charlotte, NC office)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Energy &amp; utilities, critical manufacturing, U.S. federal government/DoD, OT/IT/IoT supply chains</t>
+          <t>Critical Infrastructure cybersecurity and compliance — energy/electric utilities (NERC CIP), oil &amp; gas, healthcare (HIPAA), transportation (TSA SD02), and other critical infrastructure sectors</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Private company; size not verifiable via SEC filings (estimate: 150-400 employees based on scale of platform/funding)</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr"/>
+          <t>11-50 employees</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>$1M-$5M (estimate)</t>
+        </is>
+      </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
           <t>estimate</t>
@@ -3145,41 +3195,41 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Fortress is a well-funded, high-profile player squarely at the intersection of OT security and supply chain risk. &lt;cite index="23-19,23-20"&gt;Fortress Information Security is a cybersecurity company specializing in cyber supply chain risk management (C-SCRM) for critical infrastructure organizations and U.S. government agencies, with an AI-powered Fortress Platform enabling enterprises to identify, prioritize, assess, resolve, and continuously monitor risks across vendors, software, and hardware supply chains.&lt;/cite&gt; &lt;cite index="23-16,23-17"&gt;Fortress serves energy and utility companies, oil and gas operators, critical manufacturers, U.S. federal government agencies, and DoD contractors subject to NERC CIP, CMMC, and other critical infrastructure security regulations, with deep specialization in critical infrastructure and defense supply chain security.&lt;/cite&gt;</t>
+          <t>ITEGRITI is a boutique firm founded specifically to secure critical infrastructure, combining IT/OT cybersecurity, NERC CIP compliance, audit, and risk management services. Its leadership team includes former NERC CSO/E-ISAC Senior Director and a CEO with decades of Fortune 10 energy company IT/OT experience, making it a natural fit for OT cybersecurity advisory talent.</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Fortress has raised significant capital and expanded federal reach: &lt;cite index="29-1,29-2"&gt;Fortress Information Security announced raising $125 million from Goldman Sachs, having previously raised roughly $40 million in several funding rounds between 2015 and 2020.&lt;/cite&gt; &lt;cite index="29-13"&gt;The solution was developed in collaboration with electric utilities and the company claims it's now being used to secure 40% of the United States' power grid.&lt;/cite&gt; It continues to add partnerships, e.g., aligning with NetRise on firmware/SBOM analysis, and was recently recognized industry-wide: &lt;cite index="51-3"&gt;Fortress was named Most Innovative Critical Infrastructure Platform by The Hacker News Cybersecurity Stars Awards 2026.&lt;/cite&gt;</t>
+          <t>Company just celebrated its 10-year anniversary and highlighted growth in service lines including AI governance, Office of the CISO offerings, and an expanded 'consortium of trusted organizations' delivery model with global partners.</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Engage through its government/energy delivery and C-SCRM practice leadership; reference NAESAD/A2V data exchanges and DoD/Navy delivery work (e.g., Patuxent River SBOM analyst roles) as entry points. Active recruiting pipeline makes direct application plus LinkedIn networking with delivery/engineering leads a viable dual approach.</t>
+          <t>Target via warm introduction through advisory board members or InfraGard/ASIS network connections; highlight NERC CIP/critical infrastructure audit and vCISO experience; engage around thought-leadership content (blog, Inc. 5000 recognition) and recent 10-year anniversary momentum.</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>VP Government Delivery; Director C-SCRM Services; VP Product Security; Director OT/ICS Supply Chain Risk</t>
+          <t>Chief Delivery Officer; VP OT/ICS Cybersecurity; Director Critical Infrastructure Advisory; Practice Lead NERC CIP Compliance; Senior Manager Cybersecurity and Compliance</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Fortress Information Security OT; Fortress C-SCRM; Fortress NAESAD; Fortress Information Security supply chain</t>
+          <t>ITEGRITI Corporation; NERC CIP consultant Houston; OT/ICS cybersecurity consultant critical infrastructure; vCISO critical infrastructure advisory; ITEGRITI cybersecurity compliance</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>Multiple job boards confirm active hiring: &lt;cite index="52-2"&gt;Fortress Information Security is currently hiring for 15 open positions in the United States&lt;/cite&gt; per Glassdoor, and &lt;cite index="56-2"&gt;ZipRecruiter has 22 Fortress Information Security jobs&lt;/cite&gt; listed, including government-delivery/SBOM analyst roles requiring active clearances.</t>
+          <t>No dedicated ITEGRITI careers page with current openings was found in search results; ZoomInfo notes possible recent job posting/layoff signals but details are masked/paywalled, so hiring activity could not be confirmed.</t>
         </is>
       </c>
       <c r="R26" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="S26" t="inlineStr">
         <is>
@@ -3188,7 +3238,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>https://www.fortressinfosec.com/careers/jobs-listing</t>
+          <t>https://itegriti.com/about/</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3198,109 +3248,6 @@
       </c>
       <c r="V26" t="inlineStr"/>
       <c r="W26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Honeywell International Inc. (Honeywell OT Cybersecurity)</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>https://www.honeywell.com/us/en/company/ot-cybersecurity</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>OEM/Industrial Automation Vendor with Dedicated OT Cybersecurity Practice</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Charlotte, North Carolina, USA</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Cross-sector critical infrastructure (energy, chemicals, water, manufacturing, transportation, building automation) — Honeywell markets its OT cybersecurity practice across all 16 CISA-designated critical infrastructure sectors</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Large multinational (100,000+ employees, public company)</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>public-company (see EDGAR)</t>
-        </is>
-      </c>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J27" s="3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>Honeywell operates a dedicated, large-scale OT cybersecurity business line with 20+ years of industrial cybersecurity consulting history. Honeywell offers over 30 OT cybersecurity services designed to help customers protect continuous operations, and its team has helped hundreds of industrial companies improve OT network and asset protection over the last 20 years. It was also named a leader in the first Omdia OT Managed Cybersecurity Services report, reflecting deep market credibility for advisory/consulting talent.</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>Honeywell is actively expanding its OT cybersecurity product/service portfolio: it recently launched Honeywell Cyber Proactive Defense and an OT Security Operations Center at its 2025 Honeywell Users Group event, and published a 2025 Cyber Threat Report noting ransomware attacks targeting industrial operators jumped 46% in Q1 2025. It also runs an ongoing OT Cybersecurity Symposium series (e.g., a Dec. 2025 event in Ontario, Canada) to engage customers on cybersecurity strategy, and is investing in AI-enabled OT threat detection and post-quantum cryptography readiness content — all signals of a growing, well-funded OT security business unit.</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>Target Honeywell Building Automation, Honeywell Connected Enterprise (HCE), and Honeywell Process Solutions cybersecurity teams directly, since OT security roles are distributed across these business units rather than a single centralized group. Reference specific Honeywell offerings (Cyber Insights, Cyber Proactive Defense, AMIR, SMX) in outreach to demonstrate familiarity with their product/service stack. Engage via LinkedIn with people posting about the Honeywell Cyber Threat Report or HUG conference sessions, and consider attending/networking at Honeywell's OT Cybersecurity Symposium events.</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>VP/Director OT Cybersecurity; Global Director Cybersecurity Sales; Director Product Cyber Security; Enterprise OT Cybersecurity Leader; Director Cybersecurity Consulting Services; Sr. Director, Product Cyber Security (Chief Product Security Leader)</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>Honeywell OT Cybersecurity; Honeywell Cyber Insights; Honeywell Advanced Monitoring Incident Response; Honeywell Cybersecurity Consulting; Honeywell Connected Enterprise Security; Honeywell Building Automation OT Security</t>
-        </is>
-      </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>Active OT/cybersecurity-related job postings found across multiple boards, including a Senior Cyber Security Specialist (OT Security) role in the Netherlands within Honeywell Building Automation, Senior/Lead Cyber Security Architect/Engineer roles (Atlanta, Charlotte, Morris Plains), Enterprise OT Cybersecurity Leader (Houston), Global Director Cybersecurity Sales (Atlanta), and Senior Advanced Cloud Security Architect for Honeywell Connected Enterprise. Glassdoor shows 21 open positions and LinkedIn lists hundreds of cybersecurity-tagged roles company-wide as of research date.</t>
-        </is>
-      </c>
-      <c r="R27" t="n">
-        <v>9</v>
-      </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>AI research (verify)</t>
-        </is>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>https://www.honeywell.com/us/en/company/ot-cybersecurity</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="V27" t="inlineStr"/>
-      <c r="W27" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3313,7 +3260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3416,19 +3363,19 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Adjacent/competing service line — used heavily for niche cybersecurity, managed security, and OT-focused technical services offered by Accenture and its rivals (Deloitte, IBM, Booz Allen, etc.)</t>
+          <t>Competitor/adjacent — covers niche/specialized cybersecurity offerings such as penetration testing, incident response, and disaster recovery that overlap with OT security engagements</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>541690</t>
+          <t>561621</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Other Scientific and Technical Consulting Services</t>
+          <t>Security Systems Services (except Locksmiths)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -3438,19 +3385,19 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Adjacent service provider — covers OT/industrial risk, engineering, and specialized technical consulting used by cybersecurity consultancies for federal/industrial contracts</t>
+          <t>Adjacent service provider — physical and industrial security systems integration firms that increasingly bundle OT/ICS network security monitoring</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>561621</t>
+          <t>334513</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Security Systems Services (except Locksmiths)</t>
+          <t>Instruments and Related Products Manufacturing for Measuring, Displaying, and Controlling Industrial Process Variables</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -3460,19 +3407,19 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Adjacent physical/OT security overlap — installation, monitoring, and integration of network-connected industrial security systems (cameras, access control, SCADA-adjacent physical security)</t>
+          <t>Manufacturer served — makers of ICS/SCADA field instrumentation and process control equipment (e.g., Honeywell, Emerson, Siemens) that are core clients/partners for OT cybersecurity advisory</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>511210</t>
+          <t>335314</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Software Publishers</t>
+          <t>Relay and Industrial Control Manufacturing</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3482,19 +3429,19 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Supplier/vendor — OT security software and platform vendors (e.g., Claroty, Dragos, Nozomi Networks, Tenable.ot) whose products Accenture integrates or partners with</t>
+          <t>Manufacturer served — producers of industrial relays and control systems (e.g., Rockwell Automation, Schneider Electric) whose OT environments require cybersecurity hardening</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>334513</t>
+          <t>221100</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Instruments and Related Products Manufacturing for Measuring, Displaying, and Controlling Industrial Process Variables</t>
+          <t>Electric Power Generation, Transmission and Distribution</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -3504,19 +3451,19 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Manufacturer served — producers of industrial control system (ICS/SCADA) hardware that require OT cybersecurity hardening</t>
+          <t>Client industry — utilities are a top vertical for OT/ICS cybersecurity consulting due to critical infrastructure regulation (NERC CIP)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>221122</t>
+          <t>324110</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Electric Power Distribution</t>
+          <t>Petroleum Refineries</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -3526,19 +3473,19 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Client/manufacturer served — utilities are a top-tier OT cybersecurity client segment (grid, substation, and SCADA protection)</t>
+          <t>Client industry — oil &amp; gas refining operations rely heavily on OT/ICS security for process control and safety systems</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>324110</t>
+          <t>325110</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Petroleum Refineries</t>
+          <t>Petrochemical Manufacturing</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -3548,19 +3495,19 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Client served — critical infrastructure sector with heavy reliance on OT/ICS cybersecurity for refining and pipeline operations</t>
+          <t>Client industry — chemical/petrochemical plants are major consumers of OT cybersecurity risk assessments and IEC 62443 compliance work</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>325</t>
+          <t>511210</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Chemical Manufacturing</t>
+          <t>Software Publishers</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -3570,19 +3517,19 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Client served — process manufacturing sector requiring ICS/OT security for DCS and safety instrumented systems</t>
+          <t>Competitor/vendor — OT-focused cybersecurity software companies (e.g., Dragos, Claroty, Nozomi Networks, Tenable.ot) that partner with or compete against consulting firms like Accenture</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>336</t>
+          <t>518210</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Transportation Equipment Manufacturing</t>
+          <t>Data Processing, Hosting, and Related Services</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -3592,19 +3539,19 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Client served — automotive/aerospace manufacturers with connected factory floors (Industry 4.0) needing OT security consulting</t>
+          <t>Adjacent service provider — managed security services providers and SOC/MSSP operators delivering monitoring for OT networks</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>541511</t>
+          <t>541690</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Custom Computer Programming Services</t>
+          <t>Other Scientific and Technical Consulting Services</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -3614,51 +3561,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Competitor/adjacent — software development firms building secure OT/IT integration tools, often competing for the same consulting engagements</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>928110</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>National Security</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Secondary</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Client/government sector — federal and defense OT cybersecurity contracts (e.g., Accenture Federal Services) tied to national security infrastructure</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>541715</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Research and Development in the Physical, Engineering, and Life Sciences</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Secondary</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Adjacent service provider — engineering R&amp;D firms supporting industrial control system security research and standards development (e.g., IEC 62443)</t>
+          <t>Adjacent service provider — engineering and industrial-process consulting firms that intersect with OT cybersecurity through safety/process control advisory work</t>
         </is>
       </c>
     </row>
@@ -3760,7 +3663,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>2026-07-09T14:16:54.802556+00:00</t>
+          <t>2026-07-09T14:31:06.929479+00:00</t>
         </is>
       </c>
     </row>
@@ -3772,7 +3675,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Accenture is classified primarily as a management/IT consulting firm. Business data providers consistently list Accenture under NAICS 541618 (Other Management Consulting Services), with related entities like Accenture Federal Services under 541611 (Administrative Management and General Management Consulting Services), and broader industry rollups under 5416 (Management, Scientific, and Technical Consulting Services). For its technology/cybersecurity delivery arm, 541512 (Computer Systems Design Services) is the most commonly cited primary code for firms offering OT/IT cybersecurity consulting, since there is no single NAICS code exclusively for cybersecurity. Secondary codes reflect (1) competitor consultancies and system integrators (541519, 541511, 541690), (2) OT security software/hardware vendors and physical security integrators that Accenture partners with or competes against (511210, 561621), (3) critical-infrastructure and manufacturing client sectors that consume OT cybersecurity services — utilities, oil &amp; gas, chemicals, and industrial equipment manufacturers (221122, 324110, 325, 334513, 336) — and (4) government/defense-related codes (928110) relevant to Accenture Federal Services' OT/ICS security work. Multiple sources confirm there is no NAICS code exclusively for cybersecurity, with 541512 and 541519 being the most frequently used classifications industry-wide, supplemented by 541611 for risk/compliance consulting engagements.</t>
+          <t>Accenture is officially classified across several overlapping NAICS consulting codes depending on the business unit: 541512 (Computer Systems Design Services) is used by Accenture Federal Services/Accenture National Security Services for technology and cybersecurity consulting work, while 541611 (Administrative Management and General Management Consulting) and 541618 (Other Management Consulting Services) are used at various Accenture locations for broader management/business consulting — reflecting Accenture's blended technology-plus-strategy consulting model. There is no single NAICS code exclusively for cybersecurity or OT security; industry guidance confirms cybersecurity consulting activities are split mainly between 541512 (systems design/integration/cybersecurity consulting) and 541519 (niche services like penetration testing and incident response). For an OT cybersecurity practice specifically, secondary codes were selected to capture: (1) direct competitors and adjacent IT/physical security service providers (541519, 561621, 518210, 541690), (2) software vendors building OT-specific security tools that Accenture partners with or competes against (511210), and (3) the client-side industries and equipment manufacturers most reliant on OT cybersecurity — electric utilities, oil &amp; gas, petrochemicals, and industrial control/instrumentation manufacturers (221100, 324110, 325110, 334513, 335314), since NAICS classification of critical infrastructure sectors is explicitly used to tailor OT/ICS cybersecurity strategies and compliance frameworks like IEC 62443.</t>
         </is>
       </c>
     </row>

</xml_diff>